<commit_message>
nouveau programme.json - Lab
</commit_message>
<xml_diff>
--- a/Lab/Programme.json_builder/work/enriched.xlsx
+++ b/Lab/Programme.json_builder/work/enriched.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,7 +538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-02-04</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>La vie après Siham</t>
+          <t>Les échos du passé</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -559,73 +559,85 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Namir Abdel Messeeh</t>
+          <t>Mascha Schilinski</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Invité ADRC Cédric Lépine - Partenariat ADRC</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>Prix du jury Cannes 2025</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Prix du jury Cannes 2025</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/38/18/38181f1fe67de6a511e5a075587f98a6.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/16/07/1607b1aa4e7516d75f83006f89c4cb20.jpg</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Namir et sa mère s’étaient jurés de refaire un film ensemble, mais la mort de Siham vient briser cette promesse. Pour tenir parole, Namir plonge dans l’histoire romanesque de sa famille. Cette enquête faite de souvenirs intimes et de grands films égyptiens se transforme en un récit de transmission joyeux et lumineux, prouvant que l’amour ne meurt jamais.</t>
+          <t>Quatre jeunes filles à quatre époques différentes. Alma, Erika, Angelika et Lenka passent leur adolescence dans la même ferme, au nord de l’Allemagne. Alors que la maison se transforme au fil du siècle, les échos du passé résonnent entre ses murs. Malgré les années qui les séparent, leurs vies semblent se répondre.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Documentaire</t>
+          <t>Drame</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>155</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>France, Egypt</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Siham Abdel Messeeh, Waguih Abdel Messeeh, Nermine Abdel Messeeh, Namir Abdel Messeeh</t>
+          <t>Luise Heyer, Lena Urzendowsky, Claudia Geisler-Bading, Lea Drinda, Hanna Heckt, Laeni Geiseler, Florian Geißelmann, Andreas Anke</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Invité ADRC Cédric Lépine - Partenariat ADRC</t>
+          <t>Prix du jury Cannes 2025, Festival de Cannes 2025: Prix du Jury</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr"/>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=O-jgGbvLgVo</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000023001.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=325123.html</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>["https://fr.web.img6.acsta.net/img/79/f6/79f6b79d81860c1d4cbb675e798e9c51.jpg", "https://fr.web.img6.acsta.net/img/11/d8/11d861d6f9d1a9a192534451c63aebfe.jpg", "https://fr.web.img6.acsta.net/img/20/2d/202d9475494d01d68afe9b192758fe6a.jpg", "https://fr.web.img4.acsta.net/img/20/e0/20e02fcbc855e9ac56c7e0e5b2af9083.jpg", "https://fr.web.img3.acsta.net/img/f2/55/f255c874fd57a8cd0695819635f5dfef.jpg", "https://fr.web.img5.acsta.net/img/6a/8b/6a8b3e37794df33406364b124212c25e.jpg"]</t>
+          <t>["https://fr.web.img3.acsta.net/img/86/d3/86d38c6dd4000621947c32b2014372f3.jpg", "https://fr.web.img2.acsta.net/img/be/c5/bec52dc5aeea9924834d5f46cd9b8cc9.jpg", "https://fr.web.img6.acsta.net/img/6d/07/6d078fd7f3d7326d1c3ee3953f9bc9d1.jpg", "https://fr.web.img2.acsta.net/img/5c/db/5cdb07e0ee44ccc8941753c17d1e36a8.jpg", "https://fr.web.img5.acsta.net/img/40/d2/40d290c211e1bb18d48d917d0ca50f9b.jpg", "https://fr.web.img5.acsta.net/img/07/73/07735cd34fa049081e34c640d97fe19d.jpg", "https://fr.web.img2.acsta.net/img/f2/b4/f2b4b9064e0c0860d0a897904fbd0bf4.jpg", "https://fr.web.img4.acsta.net/img/6c/42/6c424327f43349499b27fd96f15be722.jpg", "https://fr.web.img6.acsta.net/img/85/92/8592629bc839a2ed6132c6a2898bd64e.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -635,41 +647,45 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Baise-en-ville</t>
+          <t>Christy and his brother</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>VF</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CM1</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Martin Jauvat</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Invité ADRC Chloé Caye</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>Brendan Canty</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Coip de cœur</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/8e/a5/8ea5ebba183c85d8c42b36a96b66d517.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/88/62/8862127888090061db98a62f1680fd52.jpg</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Quand sa mère menace de le virer du pavillon familial s’il ne se bouge pas les fesses, Sprite se retrouve coincé dans un paradoxe : il doit passer son permis pour trouver un taf, mais il a besoin d'un taf pour payer son permis. Heureusement, Marie-Charlotte, sa monitrice d'auto-école, est prête à tout pour l'aider - même à lui prêter son baise-en-ville. Mais... C'est quoi, au fait, un baise-en-ville ?</t>
+          <t>Expulsé de sa famille d’accueil, Christy, 17 ans, débarque chez son demi-frère, jeune papa, qu’il connait peu. Ce dernier vit mal cet arrangement qu’il espère temporaire, mais Christy se sent vite chez lui, dans ce quartier populaire de Cork, se faisant des amis et renouant avec la famille de sa mère. Les deux frères vont devoir se confronter à leur passé tumultueux pour envisager un avenir commun.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Comédie</t>
+          <t>Drame</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -679,44 +695,40 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Ireland, United Kingdom</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Martin Jauvat, Emmanuelle Bercot, William Lebghil, Anaïde Rozam, Sébastien Chassagne, Annabelle Lengronne, Michel Hazanavicius, Jérôme Niel</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Invité ADRC Chloé Caye, Fondation Gan pour le cinéma 2024: Fondation Gan - Prix à la création</t>
-        </is>
-      </c>
+          <t>Danny Power, Diarmuid Noyes, Emma Willis, Alison Oliver, Helen Behan, Chris Walley, Kane O'Connell Flynn, Ciaran Bermingham</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=6CxCD9j5GBQ</t>
+          <t>https://www.youtube.com/watch?v=yz9t81MXyt0</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000004512.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000019314.html</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>["https://fr.web.img4.acsta.net/img/5f/fd/5ffdcbf01ced3064d847cf45f68f1e8c.jpg", "https://fr.web.img2.acsta.net/img/70/8d/708dafa0d7a642ba2daf451bddddf05f.jpg", "https://fr.web.img2.acsta.net/img/ae/2b/ae2b79db000bb6e752a33401378e5b4b.jpg"]</t>
+          <t>["https://fr.web.img3.acsta.net/img/81/8e/818eeea254d15ea4716b00236a0918bd.jpg", "https://fr.web.img4.acsta.net/img/b5/5f/b55faaf266f267a80ed33293c62c4433.jpg", "https://fr.web.img6.acsta.net/img/e1/77/e17706fcba04a53a1edd40b0a02b1602.jpg", "https://fr.web.img2.acsta.net/img/44/ca/44ca7eca8532911c18bb517e8d44a57a.jpg", "https://fr.web.img5.acsta.net/img/37/21/372151cf69d85927e75aa87f32909301.jpg", "https://fr.web.img6.acsta.net/img/8b/38/8b38eb824aa3cd56fa2c21b9e97aa8a3.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -726,7 +738,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>La pire mère au monde</t>
+          <t>Ma frère</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -737,25 +749,29 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pierre Mazingarbe</t>
+          <t>Lise Akoka, Romane Gueret</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Séance EPHAD HANDI</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
+          <t>Séance EPHAD HANDI - Famille</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Tarif Unique 5 €</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/c_310_420/img/ea/fd/eafdfac8bc40d63ec84a32063363565a.jpg</t>
+          <t>https://fr.web.img5.acsta.net/c_310_420/img/35/23/35233aa3767ab31d242ec1c3ff34497c.jpg</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Louise de Pileggi, brillante substitut du procureur, a toujours eu des relations compliquées avec sa mère Judith qu’elle n’a pas vue depuis 15 ans. Quand elle se retrouve mutée au petit tribunal où Judith est greffière, Louise devient la cheffe de sa mère. Et pire encore : elles vont devoir collaborer dans une affaire à première vue banale, mais qui va mettre leurs nerfs à vif.</t>
+          <t>Shaï et Djeneba ont 20 ans et sont amies depuis l’enfance. Cet été-là, elles sont animatrices dans une colonie de vacances. Elles accompagnent dans la Drôme une bande d’enfants qui, comme elles, ont grandi entre les tours de la Place des Fêtes à Paris. À l’aube de l’âge adulte, elles devront faire des choix pour dessiner leur avenir et réinventer leur amitié.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -765,7 +781,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>112</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -775,35 +791,35 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Louise Bourgoin, Muriel Robin, Florence Loiret Caille, Sébastien Chassagne, Gustave Kervern, Patrick Descamps, Anne Benoît, Johann Cuny</t>
+          <t>Fanta Kebe, Shirel Nataf, Zakaria-Tayeb Lazab, Mouctar Diawara, Idir Azougli, Yuming Hey, Suzanne De Baecque, Amel Bent</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=DubZRp9QwsI</t>
+          <t>https://www.youtube.com/watch?v=53BgM9euEOQ</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=279638.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000007387.html</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>["https://fr.web.img4.acsta.net/img/fe/6a/fe6a2d1825f27579b5d5935d1662104f.jpg", "https://fr.web.img3.acsta.net/img/e3/d7/e3d7b58df0f285df881f289cb700433d.jpg", "https://fr.web.img2.acsta.net/img/4a/84/4a844cac98b2225c6a14af1700e6364b.jpg", "https://fr.web.img5.acsta.net/img/0b/e0/0be032fed7ca132697a0236a7442c00d.jpg", "https://fr.web.img2.acsta.net/img/0a/24/0a24e5bb15c4a635d0e3c405676d89b9.jpg", "https://fr.web.img3.acsta.net/img/44/40/444070ee5a8b27c077b983c32e328e95.jpg", "https://fr.web.img6.acsta.net/img/ee/14/ee1484bc856187e7bf54eb4fbc174baf.jpg", "https://fr.web.img5.acsta.net/img/c5/bf/c5bfdaba870ea3b8d87591a083f65456.jpg", "https://fr.web.img6.acsta.net/img/84/69/846975d92773ae0155e3482afb5b4b7f.jpg", "https://fr.web.img2.acsta.net/img/f7/a5/f7a5493041d5a798c783b71a27d026d5.jpg", "https://fr.web.img6.acsta.net/img/5d/b2/5db2f573ff0656b97aff4e839aa30813.jpg", "https://fr.web.img2.acsta.net/img/55/c3/55c32fa89f9070f778c0b90141ff9a1d.jpg", "https://fr.web.img2.acsta.net/img/f0/af/f0af70e4e07ef7f8732123cf6129a461.jpg", "https://fr.web.img5.acsta.net/img/c4/52/c45239fce1251f2373fdec9facf110e0.jpg", "https://fr.web.img4.acsta.net/img/c4/d6/c4d6d97e38ef1575d1183be1e33620bf.jpg", "https://fr.web.img2.acsta.net/img/c5/6c/c56c7f470fc89e634f8c8b8c04da0510.jpg", "https://fr.web.img5.acsta.net/img/b4/13/b4133a66dc6e338546c3df28d75ccf78.jpg"]</t>
+          <t>["https://fr.web.img3.acsta.net/img/98/b8/98b83a6cafcd5ae0c8a89c20f9ae7437.jpg", "https://fr.web.img2.acsta.net/img/37/9d/379dbf504a6aee9a25b25e1c699b25c3.jpg", "https://fr.web.img4.acsta.net/img/5e/08/5e08b0482694b6ce002742071afe0b45.jpg", "https://fr.web.img6.acsta.net/img/2d/c0/2dc0c49d0be726b94b67121cac743537.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -813,181 +829,185 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Victor comme tout le monde</t>
+          <t>Hamnet</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Chloé Zhao</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Avant-Première en Compétition</t>
+          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://fr.web.img3.acsta.net/c_310_420/img/17/7a/177a42854bab65ac4e585d4064bc3bee.jpg</t>
+          <t>https://fr.web.img2.acsta.net/c_310_420/img/9a/f5/9af5f87b39938fec50f86c32c3d31b69.jpg</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Habité par Victor Hugo, le comédien Robert Zucchini traîne une douce mélancolie lorsqu'il n'est pas sur scène. Chaque soir, il remplit les salles en transmettant son amour des mots. Jusqu’au jour où réapparaît sa fille, qu’il n’a pas vue grandir… Et si aimer, pour une fois, valait mieux qu’admirer ?</t>
+          <t>Angleterre, 1580. Un professeur de latin fauché, fait la connaissance d’Agnes, jeune femme à l’esprit libre. Fascinés l’un par l’autre, ils entament une liaison fougueuse avant de se marier et d’avoir trois enfants. Tandis que Will tente sa chance comme dramaturge à Londres, Agnes assume seule les tâches domestiques. Lorsqu’un drame se produit, le couple, autrefois profondément uni, vacille. Mais c’est de leur épreuve commune que naîtra l’inspiration d’un chef d’œuvre universel.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Comédie dramatique</t>
+          <t>Drame</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>125</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United Kingdom, United States of America</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Fabrice Luchini, Chiara Mastroianni, Louise Orry-Diquéro, Suzanne De Baecque, Marie Narbonne, Lauretta Trefeu, Iris Bry, Naidra Ayadi</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+          <t>Jessie Buckley, Paul Mescal, Emily Watson, Joe Alwyn, Jacobi Jupe, Noah Jupe, Bodhi Rae Breathnach, Olivia Lynes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026, Golden Globes 2026: Meilleur film dramatique, Meilleure actrice dans un drame</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=t0RrVuOml0M</t>
+          <t>https://www.youtube.com/watch?v=xYcgQMxQwmk</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000021956.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=315003.html</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>["https://fr.web.img4.acsta.net/img/e9/87/e987439316c89fa9fecbc48c10843d0a.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/db/27/db27c1195bfb8835aef4671ac165e436.jpg", "https://fr.web.img3.acsta.net/img/ea/c4/eac4203c2df8347475f77ec8ce61d7ca.jpg", "https://fr.web.img6.acsta.net/img/7e/b8/7eb8bf6fa577347479dfd6347f103afb.jpg", "https://fr.web.img4.acsta.net/img/b0/3d/b03d7554c97c3f7ba8c880de57c35b31.jpg", "https://fr.web.img2.acsta.net/img/e0/f2/e0f2b4497faaf505ab30ecd733f2a531.jpg", "https://fr.web.img6.acsta.net/img/9a/fd/9afde980a6402b830c5007cc66e72aff.jpg", "https://fr.web.img5.acsta.net/img/ce/fe/cefe5da862eb8228d3bf79a068a9844a.jpg", "https://fr.web.img4.acsta.net/img/c0/41/c041a05c78908f57f777fb269f515979.jpg", "https://fr.web.img3.acsta.net/img/fd/f9/fdf917bfcee844d0fbd3ac41bba90997.jpg", "https://fr.web.img5.acsta.net/img/dc/88/dc886647f0301e242fd931547cd4d10e.jpg", "https://fr.web.img2.acsta.net/img/fc/d8/fcd8803be480fc3fd79f80b56597c9ba.jpg", "https://fr.web.img2.acsta.net/img/f1/de/f1deaf59daf5e4773c85bcf1702633d7.jpg", "https://fr.web.img2.acsta.net/img/5f/dc/5fdc64d7259e00568cfd5ab9344356b1.jpg", "https://fr.web.img3.acsta.net/img/19/5f/195f3ffc57720410317e2fb3d51ae61f.jpg", "https://fr.web.img2.acsta.net/img/b8/76/b876bf840dab929460f48ff0dac4d321.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Le grand Phuket</t>
+          <t>Olivia</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Liu Yaonan</t>
+          <t>Irene Iborra</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Ciné Jeunes du samedi 18h</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Tarif Unique 4,50 €</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/c9/8a/c98a620996904fb707ac74e2ee152db7.jpg</t>
+          <t>https://fr.web.img2.acsta.net/c_310_420/img/35/40/354092484a9bc5dfedb67167f9da43da.jpg</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Li Xing, 14 ans, vit dans le sud de la Chine, dans le district de Great Phuket, en pleine reconstruction. Il s'entend mal avec sa mère, qui refuse de quitter la maison familiale vouée à la destruction. Le collège où il étudie ne lui apporte que des ennuis. Un jour, il trouve un refuge souterrain où il peut échapper à sa vie d'adolescent et où d'étranges événements se produisent…</t>
+          <t>À 12 ans, Olivia voit son quotidien bouleversé du jour au lendemain. Elle va devoir s’habituer à une nouvelle vie plus modeste et veiller seule sur son petit frère Tim. Mais, heureusement, leur rencontre avec des voisins chaleureux et hauts en couleur va transformer leur monde en un vrai film d’aventure ! Ensemble, ils vont faire de chaque défi un jeu et de chaque journée un moment inoubliable.D’après le roman Olivia de Maite Carranza.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Drame, Mystère</t>
+          <t>Animation</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>98</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Belgium, Germany, France, Hong Kong</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Li Rongkun, Yang Xuan, You Junwen, Liu Huiyun, Kang Hang, Xie Zhenan, Liu Lijun, Yan Huimei</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Festival du Film d'Animation d'Annecy 2025: Prix Fondation Gan à la Diffusion</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=8gZJSKZs-to</t>
-        </is>
-      </c>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=326632.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=302424.html</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>["https://fr.web.img3.acsta.net/pictures/24/02/12/09/34/1081778.jpg", "https://fr.web.img6.acsta.net/pictures/24/02/12/09/34/1063058.jpg", "https://fr.web.img6.acsta.net/pictures/24/02/12/09/34/1049018.jpg"]</t>
+          <t>["https://fr.web.img5.acsta.net/img/68/7d/687dcf80fd39e1a57716b2d8386570a8.jpg", "https://fr.web.img3.acsta.net/img/d5/64/d5641afeb1a1642616fed8ebddb88f7f.jpg", "https://fr.web.img5.acsta.net/img/e0/9f/e09f107f2cfe985b36a15aae0a2ffcb3.jpg", "https://fr.web.img6.acsta.net/img/5c/20/5c2057cf0bbdb2994fbb4f581cac70eb.jpg", "https://fr.web.img6.acsta.net/img/5a/95/5a956d1bc8d439383efb75c8f58020a3.jpg", "https://fr.web.img6.acsta.net/img/e0/58/e05866f0898362e1ddb408a724b4bccb.jpg", "https://fr.web.img2.acsta.net/img/d1/79/d179899a0e3dcdaa15a123c96785b7e6.jpg", "https://fr.web.img6.acsta.net/img/8c/e4/8ce4f7d363e6b866184f85fbb6ba51dc.jpg", "https://fr.web.img4.acsta.net/img/18/5e/185eb0f57dc20597fcf0762ed42135b7.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>En route</t>
+          <t>Bardot</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -998,266 +1018,282 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Alexei Mironov</t>
+          <t>Alain Berliner, Elora Thevenet</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Ciné goûter JP</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Avant-Première</t>
-        </is>
-      </c>
+          <t>Ciné Documentaire du samedi 18h</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Adhérents 4 € - Autres 5 €</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/c_310_420/img/35/69/3569e5f8d0bdaf83fc6eed80f9372f9a.jpg</t>
+          <t>https://fr.web.img3.acsta.net/c_310_420/img/18/89/188956009aaf66c5f715713a92dd670a.jpg</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Qu’il est bon de parcourir le monde ou simplement découvrir son environnement… Ici ou là, nos petits aventuriers : une charmante escargote, une fratrie de lapereaux, un jeune dragon, deux sœurs hermines, un agneau dans les nuages, et un petit garçon vont cheminer, naviguer, explorer et s’entraider. Chaque jour est un nouveau chemin pour grandir, s’émerveiller et s’ouvrir au monde.Programme :- L’Escargote à Paris d'Alexei Mironov et Yulia Matrosova (Russie, 4', 2014) : C’est parti pour notre petite escargote qui décide d’aller faire le tour du Monde. Au détour de son voyage qui l’amène à Londres, à Moscou et au Mexique, elle se pose à Paris. Rien de plus enrichissant que de découvrir d’autres cultures, et, au gré des rencontres, de s’enrichir de ce que les autres peuvent nous apporter. Mais qu’il est bon aussi de rentrer chez soi et de s’apercevoir que les vrais amis, sont ceux que nous choisissons avec le cœur.- Sevanik, le petit dragon de Harutyun Tumaghyan (Arménie, 7', 2023) : Sevanik est un petit dragon vivant dans le lac Sevan. Il n’a qu’un seul ami : un nuage duveteux. Ce nuage, un peu comme un parent ou un ange, suit chacun de ses mouvements et de ses émotions. Mais un jour, Sevanik décide de s’aventurer en dehors du lac pour découvrir la Terre ferme. Il se fait piquer par un moustique. Cet incident va chambouler les deux amis, les obliger à changer leurs habitudes et modifier leur regard sur les autres.- La Balade de Mazayka de Yuri Chaika-Pronin (Russie, 4', 2023) : Le légendaire grand-père Mazaito s’est donné pour mission de sauver de la noyade tous les animaux pris par les eaux. Chantant à la barre de sa barque, il récupère lapins et loups pour leur offrir un asile sûr sur la terre ferme.- Mû et la source divine de Malin Neumann (Allemagne, 6', 2024) : Suite à une sécheresse extrême, la source divine s’est tarie et Mû décide de partir à la recherche d’eau, indispensable pour la relancer. Accompagné de son animal de compagnie, il entreprend alors un voyage jusqu’au bout du monde et jusqu’au plus haut sommet. Mais, malgré ses efforts, sa tentative échoue. Du moins le croit-il car, finalement, un évènement inattendu va redonner vie à la source.- Aller &amp; retour de Lucia Bulgheroni et Michele Greco (Italie, 9', 2025) : Aller et Retour sont deux hermines qui à l’arrivée de l’hiver vont devoir chercher de la nourriture pour survivre. Si jeune et si vulnérable, elles vont devoir faire face à un grand danger. Que se passera-t-il quand Aller sera kidnappée ? Retour devra alors se mettre en route pour sauver sa sœur.- Songe d'un petit agneau de Hamid Karimian (Iran, 5', 2015) : Un jeune agneau s’est égaré dans une forêt inquiétante. Seul et perdu, la peur le gagne… quand soudain il perçoit les douces notes de la flûte d’un berger ! Envoûté par la volupté de la musique, l’agneau se laisse alors emporter dans un voyage imaginaire et féerique dans lequel ses craintes n’ont plus de place et qui le ramène au sein de son troupeau.</t>
+          <t>Jamais vraiment dans une case, muse de cinéastes finissant par sacrifier tout à la cause animale, Brigitte Bardot est une femme libre mais sans doute incomprise. BARDOT revient sur les aspects si contradictoires de sa vie, de sa carrière artistique légendaire à sa célèbre fondation. Elle qui bouscula l’image des femmes et fut en avance sur la conscience écologique et le bien-être animal qui semblent, enfin, pour tous une évidence. Une réflexion croisée sur ce que signifie être une femme artiste, une femme libre et parfois en avance sur son temps.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Animation, Famille</t>
+          <t>Documentaire</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>France, United Kingdom</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Brigitte Bardot, Claude Lelouch, Naomi Campbell, Paul Watson, Stella McCartney, Hugo Clément, Allain Bougrain-Dubourg</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2M1zr-f7Wtk</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000031073.html</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=304625.html</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/84/47/84478d2cb4fd84519c8311ae8c84329f.jpg", "https://fr.web.img2.acsta.net/img/01/8c/018c905f1b37dea1b18c796e4bf00817.jpg", "https://fr.web.img3.acsta.net/img/b2/6a/b26a24bf510fc9eeb1f05fa534fc4877.jpg"]</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Urchin</t>
+          <t>Grand ciel</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Harris Dickinson</t>
+          <t>Akihiro Hata</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/e7/82/e782432beca8a04cea3b2dc66459c4a5.jpg</t>
+          <t>https://fr.web.img5.acsta.net/c_310_420/img/46/06/460600d5f82b83f150654089c463af9b.jpg</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>À Londres, Mike vit dans la rue, il va de petits boulots en larcins, jusqu'au jour où il se fait incarcérer. À sa sortie de prison, aidé par les services sociaux, il tente de reprendre sa vie en main en combattant ses vieux démons.</t>
+          <t>Vincent travaille au sein d’une équipe de nuit sur le chantier de Grand Ciel, un nouveau quartier futuriste. Lorsqu’un ouvrier disparaît, Vincent et ses collègues suspectent leur hiérarchie d’avoir dissimulé son accident. Mais bientôt un autre ouvrier disparait.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Drame, Comédie</t>
+          <t>Thriller, Drame</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>91</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>United Kingdom, United States of America</t>
+          <t>France, Luxembourg</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Frank Dillane, Megan Northam, Карина Химчук, Shonagh Marie, Amr Waked, Claudia Jones, Shahzad Ali, Michael Quartey</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Festival de Cannes 2025: Un Certain Regard - Prix du meilleur acteur</t>
-        </is>
-      </c>
+          <t>Damien Bonnard, Samir Guesmi, Mouna Soualem, Tudor Aaron Istodor, Ahmed Abdel Laoui, Issaka Sawadogo, Sophie Mousel, Denis Eyriey</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=4cJL6vmYOeo</t>
+          <t>https://www.youtube.com/watch?v=DkPQbmM-uZM</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000019912.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=300430.html</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>["https://fr.web.img5.acsta.net/img/bb/78/bb784f39d4843f599afba87529b2c028.jpg", "https://fr.web.img2.acsta.net/img/df/3d/df3dc86c2a96673a0d49796581ea5929.jpg", "https://fr.web.img4.acsta.net/img/1e/44/1e4451e35e6059ee33003bb1ddbe8b9c.jpg", "https://fr.web.img2.acsta.net/img/2d/a2/2da21da8e6c084f763290e30f0e31548.jpg", "https://fr.web.img6.acsta.net/img/da/30/da301edeec034ee0839592ee70672741.jpg", "https://fr.web.img4.acsta.net/img/fc/1e/fc1e3b1ba4bbd2e5fb722ed5f0b294e3.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/0f/e0/0fe0a74367803075fd0f0381d06bd4f3.jpg", "https://fr.web.img6.acsta.net/img/49/75/4975868cbec7f4b9228533568e65a83a.jpg", "https://fr.web.img4.acsta.net/img/ed/d1/edd1eaa8be28495ddb4a4ffaef01abb0.jpg", "https://fr.web.img4.acsta.net/img/09/5f/095fef1364af93787d4e13e110fb9dae.jpg", "https://fr.web.img5.acsta.net/img/f4/c2/f4c25e50a561c0566c338c5485e0d70d.jpg", "https://fr.web.img5.acsta.net/img/02/cf/02cf505e6f0ec20bfd9e08bfe041dc31.jpg", "https://fr.web.img6.acsta.net/img/c1/37/c137795561f8165a58e53498c0fe86ce.jpg", "https://fr.web.img4.acsta.net/img/ba/7e/ba7e00cac438cb9a64541afba9f3de54.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Noise</t>
+          <t>Biscuit le chien fantastique</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Soo-jin Kim</t>
+          <t>Shea Wageman</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/img/14/b1/14b1a952a540a054f5ffe0712e82ab86.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/7b/09/7b095f309baf4441fc5966b2f217900e.jpg</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Ju-young, malentendante, découvre que sa sœur a mystérieusement disparu de son appartement. En cherchant des réponses, elle se heurte à des voisins terrifiés, obsédés par le silence, et à une atmosphère de plus en plus oppressante. La nuit, des bruits inexpliqués résonnent dans l’immeuble déserté, éveillant une présence invisible. Ce qu’elle croyait être une simple disparition devient une plongée terrifiante dans un cauchemar hanté par le silence.</t>
+          <t>Danny et son petit chien Biscuit sont les meilleurs amis du monde. Un jour, une magie mystérieuse donne à Biscuit des pouvoirs incroyables : il peut désormais parler et voler. Dès que quelqu’un a besoin de lui, il met son masque, enfile sa cape et s’élance dans le ciel pour aider : il est devenu un chien fantastique ! Biscuit a désormais deux passions : manger des tacos et sauver le monde. Mais Pudding, le chat du voisin, lui aussi doté de super-pouvoirs, rêve de faire régner les chats sur l’univers. Danny et Biscuit devront prouver qu’ensemble, rien ne peut les arrêter !</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Epouvante-horreur, Thriller</t>
+          <t>Animation, Comédie, Famille</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>94</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Owen Wilson, Dawson Littman, Tabitha St. Germain, Sebastian Billingsley-Rodriguez, Rhona Rees, Anthony Bolognese, Caitlynne Medrek, Emily Delahunty</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>2023-04-14</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VmxXMWGaDzQ</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=325653.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000017117.html</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>["https://fr.web.img6.acsta.net/img/16/2e/162eb2cb9a4301b8b93a8ce08ba24416.jpg"]</t>
+          <t>["https://fr.web.img3.acsta.net/img/cc/bb/ccbb0018fbe560c8535c07949d408025.jpg", "https://fr.web.img3.acsta.net/img/e7/ac/e7acc11655324629f86345607eafcf23.jpg", "https://fr.web.img2.acsta.net/img/f9/7b/f97bfe76e783f57e01a872b7c763cf47.jpg", "https://fr.web.img5.acsta.net/img/7f/c6/7fc688f605e3c9f8bb6fe9058bc80942.jpg", "https://fr.web.img5.acsta.net/img/67/0e/670e08bbd5558a2b53def24b58a59715.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Les fleurs du manguier</t>
+          <t>L'affaire Bojarski</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Akio Fujimoto</t>
+          <t>Jean-Paul Salomé</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/img/b4/c1/b4c1790cacbd833589c6a4de26805535.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/18/05/18059e8dd9bca2e516d41023cc08d9d1.jpg</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Dans l'espoir de retrouver leur famille dispersée, Shafi, 4 ans, et sa sœur Somira, 9 ans, quittent un camp Rohingyas du Bangladesh pour rejoindre la Malaisie. Guidés par leur regard d’enfant, ils entreprennent une traversée périlleuse.</t>
+          <t>Jan Bojarski, jeune ingénieur polonais, se réfugie en France pendant la guerre. Il y utilise ses dons pour fabriquer des faux papiers pendant l’occupation allemande. Après la guerre, son absence d’état civil l’empêche de déposer les brevets de ses nombreuses inventions et il est limité à des petits boulots mal rémunérés… jusqu’au jour où un gangster lui propose d’utiliser ses talents exceptionnels pour fabriquer des faux billets. Démarre alors pour lui une double vie à l’insu de sa famille. Très vite, il se retrouve dans le viseur de l’inspecteur Mattei, meilleur flic de France.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1267,59 +1303,55 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>128</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Japan, France, Malaysia, Germany</t>
+          <t>France, Belgium</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Muhammad Shofik Rias Uddin, Shomira Rias Uddin</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Mostra de Venise 2025: Prix spécial du jury Orizzonti</t>
-        </is>
-      </c>
+          <t>Reda Kateb, Sara Giraudeau, Bastien Bouillon, Quentin Dolmaire, Pierre Lottin, Camille Japy, Lolita Chammah, Olivier Loustau</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>2025-08-31</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ZNyi9LzJkb4</t>
+          <t>https://www.youtube.com/watch?v=lz4trma4mCU</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000027824.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000014092.html</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>["https://fr.web.img4.acsta.net/img/a0/ce/a0ce92b38c457f2b9817375347c75c80.jpg", "https://fr.web.img2.acsta.net/img/3c/5a/3c5af433d706b834e7dc8a8182960a5a.jpg", "https://fr.web.img6.acsta.net/img/00/fb/00fbc4831a05563c3d66fe690b5a9d5f.jpg", "https://fr.web.img5.acsta.net/img/31/97/3197ea34f7123218da9f5b62b0233282.jpg"]</t>
+          <t>["https://fr.web.img4.acsta.net/img/15/d8/15d8fafca4998c253b2513d29f223350.jpg", "https://fr.web.img5.acsta.net/img/81/b3/81b30ddb0cecd137cedc5220f971c839.jpg", "https://fr.web.img6.acsta.net/img/b1/cf/b1cfe81aa1138030e212e9c701898bf6.jpg", "https://fr.web.img5.acsta.net/img/5a/cc/5acce5895b2080afc842c8d57340122c.jpg", "https://fr.web.img6.acsta.net/img/5d/1e/5d1e210d87c5045ba1d443e552d407f3.jpg", "https://fr.web.img6.acsta.net/img/b1/0f/b10f18819f1ccea971de115bc964d1d6.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sauvage</t>
+          <t>Tafiti</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1330,75 +1362,83 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Camille Ponsin</t>
+          <t>Nina Wels</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/img/18/1a/181a47be9ff7a00987d7387430b36139.jpg</t>
+          <t>https://fr.web.img5.acsta.net/c_310_420/img/e7/ff/e7ffdee0f33865e434c017c192af11ac.jpg</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Au cœur d’une vallée reculée des Cévennes, des néo-ruraux vivent en autarcie, ne s’interdisant rien et partageant tout. Chacun y trouve sa place, son compte, son but. Chacun, sauf Anja. Enfant insaisissable et perturbée, elle va un jour fuir pour aller vivre à l’état quasi sauvage dans les bois alentour mettant à mal le fragile équilibre de la communauté. Inspiré d’une histoire vraie.</t>
+          <t>Lorsque Tafiti, un jeune suricate, rencontre Mèchefol, un potamochère aussi sympathique qu’exubérant, il sait qu’ils ne pourront jamais devenir amis. En effet, la vie dans le désert est pleine de dangers et Tafiti a toujours respecté la règle essentielle de survie chez les suricates : il ne faut jamais se lier aux étrangers. Mais lorsque son grand-père est mordu par un serpent venimeux, Tafiti n’a pas le choix. Il doit partir à la recherche d’une fleur légendaire qui guérit de tous les maux, mais qui pousse au-delà des vastes étendues brûlantes du désert. Une quête périlleuse que Tafiti décide d’affronter seul. Mais c’est sans compter sur Mèchefol, bien décidé à accompagner son nouveau meilleur ami dans cette aventure, qu’il le veuille ou non…</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Drame</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr"/>
+          <t>Animation, Famille, Aventure</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Lou Lampros, Céline Sallette, Bertrand Belin</t>
+          <t>Cosima Henman, Steve Hudson, Bürger Lars Dietrich, Thomas Schmuckert, Dela Dabulamanzi, Simon Werner, Dustin Semmelrogge, Simone Cohn-Vossen</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr"/>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0AG59XQEhbA</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000007389.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=327254.html</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>["https://fr.web.img4.acsta.net/img/92/bf/92bf0fb31086774f583f545151103a6c.jpg"]</t>
+          <t>["https://fr.web.img5.acsta.net/img/19/77/1977bdc7a0058cac90b8d00732caf0ca.jpg", "https://fr.web.img4.acsta.net/img/52/e6/52e62dd9215f23f1e25d326ba6b7a5fa.jpg", "https://fr.web.img2.acsta.net/img/e5/7e/e57edcf31ace74fb0a0f6f4de3be14cd.jpg", "https://fr.web.img6.acsta.net/img/aa/9f/aa9ff537ce0c29024615907c2622e4eb.jpg", "https://fr.web.img2.acsta.net/img/e5/8e/e58e207ab8bc2ac27ba7fec7da0c3696.jpg", "https://fr.web.img6.acsta.net/img/0a/ff/0aff7a5c96e70c97623d4098cfe9e51b.jpg", "https://fr.web.img4.acsta.net/img/83/73/837380da5f0906bbc4ddd94b380822c0.jpg", "https://fr.web.img3.acsta.net/img/65/3e/653e66af639a0e783b18aecde51ff7f3.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>I swear</t>
+          <t>Le mage du Kremlin</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1409,73 +1449,73 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Kirk Jones</t>
+          <t>Olivier Assayas</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/c_310_420/img/1c/f8/1cf8c5c5caa2a19a90d78914da6416f7.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/27/26/27264fbe0076f4db99b28acfa0e21ac5.jpg</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>L'histoire vraie et le parcours semé d'embûches de John Davidson, un adolescent atteint du syndrome de la Tourette, une maladie encore méconnue dans les années 1980.</t>
+          <t>Russie, dans les années 1990. L’URSS s’effondre. Dans le tumulte d’un pays en reconstruction, un jeune homme à l’intelligence redoutable, Vadim Baranov, trace sa voie. D’abord artiste puis producteur de télé-réalité, il devient le conseiller officieux d’un ancien agent du KGB promis à un pouvoir absolu, le futur « Tsar » Vladimir Poutine. Plongé au cœur du système, Baranov devient un rouage central de la nouvelle Russie, façonnant les discours, les images, les perceptions. Mais une présence échappe à son contrôle : Ksenia, femme libre et insaisissable, incarne une échappée possible, loin des logiques d’influence et de domination. Quinze ans plus tard, après s’être retiré dans le silence, Baranov accepte de parler. Ce qu’il révèle alors brouille les frontières entre réalité et fiction, conviction et stratégie. Le Mage du Kremlin est une plongée dans les arcanes du pouvoir, un récit où chaque mot dissimule une faille.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Drame, Biopic</t>
+          <t>Thriller</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>145</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>United Kingdom, Ireland</t>
+          <t>France, United States of America, United Kingdom</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Robert Aramayo, Maxine Peake, Shirley Henderson, Peter Mullan, Scott Ellis Watson, Sanjeev Kohli, Ron Donachie, Steven Cree</t>
+          <t>Paul Dano, Jude Law, Alicia Vikander, Tom Sturridge, Will Keen, Jeffrey Wright, Andris Keišs, Magne-Håvard Brekke</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=oeWqQN3snCU</t>
+          <t>https://www.youtube.com/watch?v=B5iSUmP4I6E</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000009982.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000005026.html</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>["https://fr.web.img6.acsta.net/img/98/9e/989ef532221684aa7746216d15267395.jpg", "https://fr.web.img6.acsta.net/img/70/18/70189dfd2025cfd793467526b00a214e.jpg", "https://fr.web.img6.acsta.net/img/bb/28/bb28d97eb5f9d7a6490a67cbb11dcab2.jpg", "https://fr.web.img4.acsta.net/img/97/38/9738737f981755f47fac4ae5e014beb8.jpg", "https://fr.web.img2.acsta.net/img/d9/40/d9407b614190b30e0626fbd1049eae33.jpg", "https://fr.web.img3.acsta.net/img/6b/e4/6be422c2ab0c37d8d576163727d27639.jpg", "https://fr.web.img2.acsta.net/img/32/49/32494080ea26a9ab5cf160990bd16f2b.jpg", "https://fr.web.img3.acsta.net/img/ae/86/ae86246f761f58aa29eeff665daef98d.jpg", "https://fr.web.img6.acsta.net/img/7b/ff/7bff646f1cfe461e1fbe2fa0f9a5dab2.jpg", "https://fr.web.img2.acsta.net/img/8b/f7/8bf78a61a305680944e06c8e34f3a294.jpg", "https://fr.web.img6.acsta.net/img/c4/92/c49243ebe789ea388e4781f4d701c9c5.jpg", "https://fr.web.img3.acsta.net/img/24/f8/24f8601263c3732cc5c947b5472d28cc.jpg", "https://fr.web.img4.acsta.net/img/24/ef/24efce29c062578347603c1115087363.jpg", "https://fr.web.img5.acsta.net/img/01/8c/018c61a8473809bf69ffb453092d813e.jpg", "https://fr.web.img2.acsta.net/img/b3/f3/b3f32b141ab8950d111a60451cccf3dd.jpg", "https://fr.web.img6.acsta.net/img/5b/8a/5b8a3daf65b91b6f7f9f323823b25f1e.jpg", "https://fr.web.img4.acsta.net/img/f9/77/f977a3d6fffcb3d149350eecfacf3dba.jpg", "https://fr.web.img6.acsta.net/img/ff/08/ff08181aaf0e101ff247f5ee4620df45.jpg", "https://fr.web.img2.acsta.net/img/de/fb/defb2b502a2f7a0ba41042967ebfc92f.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/29/4c/294c8fa12ac7e3930bca5c716a63a0f5.jpg", "https://fr.web.img5.acsta.net/img/e1/92/e1920a60aa6ee9290fc41bc6f15bb79d.jpg", "https://fr.web.img6.acsta.net/img/46/ae/46aea80f14f96ea297a83b899f570449.jpg", "https://fr.web.img3.acsta.net/img/92/8e/928e332e5da006270382516c3782a9d2.jpg", "https://fr.web.img6.acsta.net/img/a9/61/a9617f337638540cbd0e9dd3a7f89fab.JPG", "https://fr.web.img6.acsta.net/img/2e/f7/2ef712f51779e0ff419c6a0db501e5c4.jpg", "https://fr.web.img4.acsta.net/img/4b/de/4bde2f077a644e4d421af6db418cb9e1.jpg", "https://fr.web.img3.acsta.net/img/c7/5f/c75fb2423730c53d9d2b5dfdcc972802.jpg", "https://fr.web.img3.acsta.net/img/26/de/26de415570776b334e7f6955ae682f6c.jpg", "https://fr.web.img6.acsta.net/img/09/61/0961c8b58b6254e6b50ee5835cdd2e78.jpg", "https://fr.web.img2.acsta.net/img/e8/8a/e88a07db6b466338894b271fc9685194.jpg", "https://fr.web.img4.acsta.net/img/62/06/6206da95f59ae93b7530c5384090c899.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1485,179 +1525,159 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ma frère</t>
+          <t>The mastermind</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Lise Akoka, Romane Gueret</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Prix du jury et Prix du jury presse Pauillac 2025</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+          <t>Kelly Reichardt</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/c_310_420/img/35/23/35233aa3767ab31d242ec1c3ff34497c.jpg</t>
+          <t>https://fr.web.img4.acsta.net/c_310_420/img/9b/e7/9be71377d6e8e664aa6225ee84a1daf5.jpg</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Shaï et Djeneba ont 20 ans et sont amies depuis l’enfance. Cet été-là, elles sont animatrices dans une colonie de vacances. Elles accompagnent dans la Drôme une bande d’enfants qui, comme elles, ont grandi entre les tours de la Place des Fêtes à Paris. À l’aube de l’âge adulte, elles devront faire des choix pour dessiner leur avenir et réinventer leur amitié.</t>
+          <t>Massachussetts, 1970. Père de famille en quête d'un nouveau souffle, Mooney décide de se reconvertir dans le trafic d'œuvres d'art. Avec deux complices, il s'introduit dans un musée et dérobe des tableaux. Mais la réalité le rattrape : écouler les œuvres s’avère compliqué. Traqué, Mooney entame alors une cavale sans retour.</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Comédie</t>
+          <t>Drame, Policier</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>112</t>
+          <t>110</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United Kingdom, United States of America</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Fanta Kebe, Shirel Nataf, Zakaria-Tayeb Lazab, Mouctar Diawara, Idir Azougli, Yuming Hey, Suzanne De Baecque, Amel Bent</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>Prix du jury et Prix du jury presse Pauillac 2025</t>
-        </is>
-      </c>
+          <t>Josh O'Connor, Alana Haim, Hope Davis, John Magaro, Gaby Hoffmann, Jasper Thompson, Sterling Thompson, Bill Camp</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=53BgM9euEOQ</t>
+          <t>https://www.youtube.com/watch?v=ASH5vXpi3xA</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000007387.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000012006.html</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>["https://fr.web.img3.acsta.net/img/98/b8/98b83a6cafcd5ae0c8a89c20f9ae7437.jpg", "https://fr.web.img2.acsta.net/img/37/9d/379dbf504a6aee9a25b25e1c699b25c3.jpg", "https://fr.web.img4.acsta.net/img/5e/08/5e08b0482694b6ce002742071afe0b45.jpg", "https://fr.web.img6.acsta.net/img/2d/c0/2dc0c49d0be726b94b67121cac743537.jpg"]</t>
+          <t>["https://fr.web.img2.acsta.net/img/01/46/01461c4b5cc6ef2ee6f283f387b27230.jpg", "https://fr.web.img6.acsta.net/img/d5/6a/d56a3d76132fe08b842ec450a47996ce.jpg", "https://fr.web.img6.acsta.net/img/57/ae/57ae704079ab723424601cb09d967ca2.jpg", "https://fr.web.img5.acsta.net/img/f1/af/f1afb00d14115a94ced5b55bd7696aa3.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Tatouage</t>
+          <t>Avatar De cendres et de feu</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Yasuzo Masumura</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Soirée avec Pup En Vol + invité (à préciser) - Partenariat ADRC</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>James Cameron</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Famille - 2D</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/d1/e0/d1e0f786717651d20890faeb1892977b.jpg</t>
-        </is>
-      </c>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>La jeune Otsuya et son amant Shinsuke fuient la maison familiale pour vivre leur amour et trouvent refuge chez Gonji, un escroc qui se prétend être leur ami mais il les trahit. Il vend la jeune fille au tenancier d’une maison de geishas qui fait tatouer sur le dos d’Otsuya une araignée à tête humaine dans le but de briser sa volonté. Le contraire se produit et le tatouage métamorphose Otsuya. Elle devient une geisha sans scrupule et extermine les hommes qui ont fait son malheur. Manipulatrice et sanguinaire, elle semble possédée par l’araignée gravée sur sa peau…</t>
+          <t>Après la mort de Neteyam, Jake et Neytiri affrontent leur chagrin tout en faisant face au Peuple des Cendres, une tribu Na’vi redoutable menée par le fougueux Varang, alors que le conflit sur Pandora s’intensifie et qu’une nouvelle quê morale s’amorce.</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Drame</t>
+          <t>Science-Fiction, Aventure, Fantastique</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>198</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Ayako Wakao, 長谷川明男, 山本學, 佐藤慶, 須賀不二男, Asao Uchida, 藤原礼子, 毛利菊枝</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>Soirée avec Pup En Vol + invité (à préciser) - Partenariat ADRC</t>
-        </is>
-      </c>
+          <t>Sam Worthington, Zoe Saldaña, Sigourney Weaver, Stephen Lang, Oona Chaplin, Jack Champion, Kate Winslet, Cliff Curtis</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2004-12-22</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=gb9DKq21rDA</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=25663.html</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>["https://fr.web.img3.acsta.net/pictures/22/10/03/11/59/2217050.jpg"]</t>
-        </is>
-      </c>
+          <t>https://www.youtube.com/watch?v=Zegl3vxOPjM</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1667,245 +1687,264 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A pied d'œuvre</t>
+          <t>En garde</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Valérie Donzelli</t>
+          <t>Nelicia Low</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Partenariat ADRC</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>Grand Prix du Jury La Roche sur Yon - Meilleur réalisation Karlovy Vary</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Grand Prix du Jury La Roche sur Yon - Meilleur réalisation Karlovy Vary</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/47/c1/47c1b14d006b27555c7ef261736328c2.jpg</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Achever un texte ne veut pas dire être publié, être publié ne veut pas dire être lu, être lu ne veut pas dire être aimé, être aimé ne veut pas dire avoir du succès, avoir du succès n'augure aucune fortune.
- À Pied d’œuvre raconte l'histoire vraie d'un photographe à succès qui abandonne tout pour se consacrer à l'écriture, et découvre la pauvreté.</t>
+          <t>Jie, un jeune talent prometteur de l’escrime, renoue avec son frère aîné Han, récemment libéré après sept ans de prison pour la mort accidentelle d’un adversaire lors d’une compétition. En secret, Han soutient Jie dans son entraînement, l’aidant à viser une qualification aux championnats nationaux. Mais une dispute éclate, et Jie commence à douter de l’innocence de son frère.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Comédie, Drame</t>
+          <t>Drame</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>106</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Singapore, Taiwan, Poland</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Bastien Bouillon, Marie Rivière, Virginie Ledoyen, André Marcon, Pauline Clément, Arthur Dupont, Émilie Caen, Quentin Dolmaire</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr"/>
+          <t>劉修甫, 曹佑寧, 丁寧, Rosen Tsai, 林子恆, 曾向镇, 謝以樂, 楊文文</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Grand Prix du Jury La Roche sur Yon - Meilleur réalisation Karlovy Vary</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FQgcG7I2aho</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=307013.html</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img5.acsta.net/img/1d/5e/1d5ed38ccb2c6e3caf0b7bfed8c53f9d.jpg", "https://fr.web.img6.acsta.net/img/1e/e5/1ee5361e85068cd0e11e1b154f96a940.jpg"]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Alter ego</t>
+          <t>Le gâteau du président</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>VF</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CM2</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Nicolas Charlet, Bruno Lavaine</t>
+          <t>Hasan Hadi</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/img/8e/e1/8ee1e2ac450dea02a69bf8cabb0b74a6.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/e6/19/e6195fdd0bbba065280ae124d28ea94b.jpg</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Alex a un problème : son nouveau voisin est son sosie parfait. Avec des cheveux. Un double en mieux, qui va totalement bouleverser son existence.</t>
+          <t>Dans l’Irak de Saddam Hussein, Lamia, 9 ans, se voit confier la lourde tâche de confectionner un gâteau pour célébrer l’anniversaire du président. Sa quête d’ingrédients, accompagnée de son ami Saeed, bouleverse son quotidien.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Comédie</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr"/>
+          <t>Drame</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Laurent Lafitte, Olga Kurylenko, Blanche Gardin, Valérie Donzelli, Monsieur Fraize, Zabou Breitman, Bertrand Goncalves</t>
+          <t>Banin Ahmad Nayef, Sajad Mohamad Qasem, Waheed Thabet Khreibat, Rahim AlHaj, Muthanna Malaghi, Ahmad Qasem Saywan, Thaer Salem, Fatima Abouharoon</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr"/>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8i3idbVnC6I</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=288260.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000023006.html</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>["https://fr.web.img6.acsta.net/img/6b/da/6bdaeb4a15e035b7aa58b4e87bd47ac7.jpg", "https://fr.web.img2.acsta.net/img/b9/62/b962e3314824b9b32d8cf4320496290c.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/e6/d0/e6d0d27f1ee4074bcb15c1798450bcf5.jpg", "https://fr.web.img2.acsta.net/img/01/07/010737a7656331d34031a3f11edcca0f.jpg", "https://fr.web.img5.acsta.net/img/b8/80/b880b190c52ee73455579a566f41027a.jpg", "https://fr.web.img2.acsta.net/img/b4/0f/b40f6bacb2fa739c18dd4ecdca6077e0.jpg", "https://fr.web.img5.acsta.net/img/11/69/1169a9082f16d9eff6019ffb541ca320.jpg", "https://fr.web.img3.acsta.net/img/06/c0/06c091be44fae3533e737cd30061e946.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Le mystérieux regard du flamant rose</t>
+          <t>Les toutes petites créatures 2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Diego Cespedes</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+          <t>Lucy Izzard</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Tarif Unique 3 €</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/img/53/64/53648efa9d26840b243a90d1cd2ec989.jpg</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Début des années 1980, dans le désert chilien. Lidia, 11 ans, grandit au sein d’une famille flamboyante qui a trouvé refuge dans un cabaret, aux abords d’une ville minière. Quand une mystérieuse maladie mortelle commence à se propager, une rumeur affirme qu’elle se transmettrait par un simple regard. La communauté devient rapidement la cible des peurs et fantasmes collectifs. Dans ce western moderne, Lidia défend les siens.</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Drame</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>108</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>Chile, France, Spain, Belgium, Germany</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>Tamara Cortés, Matías Catalán, Paula Dinamarca, Claudia Cabezas, Luis Dubó, Andrés Almeida, Felipe Ríos, Vicente Caballero</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition, Festival de Cannes 2025: Prix Un Certain Regard</t>
-        </is>
-      </c>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/70/e4/70e4bca25a2fa64e3574bcb887805ffe.jpg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>2025-05-15</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=UscRzx6i53M</t>
-        </is>
-      </c>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=298832.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000037794.html</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>["https://fr.web.img2.acsta.net/img/82/90/82907cef76c8a8ed8ab5d99aab91f455.jpg", "https://fr.web.img2.acsta.net/img/44/85/44856197be75652c1527a3fcfc6a3d8b.jpg", "https://fr.web.img4.acsta.net/img/51/ab/51abdf1a07284b46031cdcda424d365e.jpg", "https://fr.web.img3.acsta.net/img/d3/3f/d33f7ebf1c5fefeb979bbd0439b138d0.png"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/20/9f/209f6648709f5ac9ac1b24d0b7300e8b.jpg", "https://fr.web.img6.acsta.net/img/e9/8d/e98d3ea0f91318eae342f1679376a5f5.jpg", "https://fr.web.img4.acsta.net/img/25/42/2542406b179eaa94973416ee53983824.jpg", "https://fr.web.img2.acsta.net/img/b4/be/b4bee561b2baf9b5ce48442ab59426f0.jpg", "https://fr.web.img6.acsta.net/img/95/4f/954f8835a08c41b04a5c95b7651eb3ef.jpg", "https://fr.web.img4.acsta.net/img/51/08/5108a7f9bd7a372c10b97486344b08c4.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Un jour avec mon père</t>
+          <t>Nuages flottants</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1916,112 +1955,116 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Akinola Davies</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Séance avancée pour jurys - pas dans prog</t>
-        </is>
-      </c>
+          <t>Mikio Naruse</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Ciné Patrimoine du samedi 18h</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Adhérents 4 € - Autres 5 €</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/3a/17/3a17a236cc7eb6ab8b568027211f5224.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/1a/71/1a7161c2d9b100af2aaa05b060e14945.jpg</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Un jour avec mon père est un récit semi-autobiographique se déroulant sur une seule journée dans la mégalopole nigériane, Lagos, pendant la crise électorale de 1993. Un père tente de guider ses deux jeunes fils à travers l'immense ville alors que des troubles politiques menacent.</t>
+          <t>Après la défaite japonaise, Yukiko, dactylographe sans le sou, retourne à Tokyo dans l’espoir de renouer avec Tomioka, un homme marié avec qui elle a vécu une intense histoire d’amour en Indochine durant la Seconde Guerre mondiale. Mais si leurs retrouvailles ravivent les braises de cette ancienne passion qui les hante, le sombre et indécis Tomioka ne semble pas partager les espoirs de Yukiko. Luttant pour survivre dans une société dévastée, la jeune femme emploiera toutes ses forces à le reconquérir...</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Drame</t>
+          <t>Drame, Romance</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>124</t>
         </is>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition, Festival de Cannes 2025: Caméra d'Or - Mention spéciale</t>
-        </is>
-      </c>
+      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr"/>
+          <t>1984-01-25</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=26e44cJ1G5Y</t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000019740.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1930.html</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>["https://fr.web.img2.acsta.net/img/9d/c8/9dc8a396dd653369fa38f649ce901b6c.jpg", "https://fr.web.img4.acsta.net/img/fc/c2/fcc2c65af7e14662b883a61b7ee9c6a4.jpg", "https://fr.web.img6.acsta.net/img/4c/13/4c136a85f4474c6e13b28af2437902c7.jpg"]</t>
+          <t>["https://fr.web.img5.acsta.net/img/30/4e/304ec21c6636d0f0368e3cf0b959f6bc.jpg", "https://fr.web.img6.acsta.net/img/cb/37/cb37f6c5895a53951c3c065005ce05f2.jpg", "https://fr.web.img6.acsta.net/img/27/20/2720359df0f6172141b00af19d329b71.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Maspalomas</t>
+          <t>Palestine 36</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Aitor Arregi, José Mari Goenaga</t>
+          <t>Annemarie Jacir</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>AP-COMP  Prix Cinema Europa Les Arcs 2025, Prix d'interprétation San Sebastian 2025</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>Grand Prix Tokyo - Meilleur film Milan</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Partenariat Festival DIAM</t>
+          <t>Grand Prix Tokyo - Meilleur film Milan</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/img/bc/e6/bce6ba592dc6197d53f2b4234b3318b5.jpg</t>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/37/0c/370c9b5f7f8502fb80051e5e9920fe9b.jpg</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Vicente, un vieil homme ouvertement homosexuel qui, lorsqu'il est admis dans une maison de retraite, décide de cacher son orientation sexuelle.</t>
+          <t>Palestine, 1936. La grande révolte arabe, destinée à faire émerger un État indépendant, se prépare alors que le territoire est sous mandat britannique.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2031,59 +2074,59 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>119</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Palestinian Territory, United Kingdom, France, Denmark, Qatar</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>José Ramón Soroiz, Nagore Aranburu, Kandido Uranga, Zorion Eguileor, Kepa Errasti, Cristina Yélamos, Ana Elordi, Miren Gaztañaga</t>
+          <t>كريم داود عناية, Yasmine Al Massri, Billy Howle, Dhafer L'Abidine, Ward Helou, Robert Aramayo, Yafa Bakri, Wardi Eilabouni</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>AP-COMP  Prix Cinema Europa Les Arcs 2025, Prix d'interprétation San Sebastian 2025</t>
+          <t>Grand Prix Tokyo - Meilleur film Milan</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2025-10-06</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=8o6gkyinORg</t>
+          <t>https://www.youtube.com/watch?v=7azScdJHB_A</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000017160.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000022541.html</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>["https://fr.web.img6.acsta.net/img/c9/9f/c99f11251f18674fd2b7a422d0691ff8.jpg", "https://fr.web.img3.acsta.net/img/7a/46/7a469765f8608f20460ab2bb2ebca382.jpg", "https://fr.web.img5.acsta.net/img/9e/3a/9e3a25b3bb74c9d42d4690716b5ed194.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/32/c9/32c950d9134bd15520ba8979e8dd1e83.jpg", "https://fr.web.img5.acsta.net/img/9e/9b/9e9ba1c64e61b67287fedecbb0fc951d.jpg", "https://fr.web.img6.acsta.net/img/87/86/8786dbb2eb68ac00ab806e70114a63c1.jpg", "https://fr.web.img5.acsta.net/img/51/76/5176ce9562ceda7efd0ed448ea705d08.jpg", "https://fr.web.img6.acsta.net/img/72/33/72333e39f472f5d3aa5f1bfef49f8d59.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>La danse des renards</t>
+          <t>Le chant des forêts</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2094,166 +2137,170 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Valéry Carnoy</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Repas partagé entres les 2 films 19h45</t>
-        </is>
-      </c>
+          <t>Vincent Munier</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Documentaire Famille</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Tarif Unique 4,50 €</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/img/0b/dc/0bdccf730ab568608d09d272f722d91b.jpg</t>
+          <t>https://fr.web.img2.acsta.net/c_310_420/img/f5/52/f5523e15c97af96169bdc93479553602.jpg</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Dans un internat sportif, Camille, un jeune boxeur virtuose, est sauvé in extremis d’un accident mortel par son meilleur ami Matteo. Alors que les médecins le pensent guéri, une douleur inexpliquée l’envahit peu à peu, jusqu’à remettre en question ses rêves de grandeur.</t>
+          <t>Après La Panthère des neiges, Vincent Munier nous invite au coeur des forêts des Vosges. C’est ici qu’il a tout appris grâce à son père Michel, naturaliste, ayant passé sa vie à l’affut dans les bois. Il est l’heure pour eux de transmettre ce savoir à Simon, le fils de Vincent. Trois regards, trois générations, une même fascination pour la vie sauvage. Nous découvrirons avec eux cerfs, oiseaux rares, renards et lynx… et parfois, le battement d’ailes d’un animal légendaire : le Grand Tétras.</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Drame</t>
+          <t>Documentaire</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>93</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Belgium, France</t>
+          <t>France</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Samuel Kircher, Faycal Anaflous, Jef Jacobs, Anna Heckel, Jean-Baptiste Durand, Hassane Alili, Salahdine El Garchi, Yoann Blanc</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+          <t>Vincent Munier, Michel Munier, Simon Munier</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>2025-05-17</t>
+          <t>2025-12-17</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xdSNIPsLoug</t>
+          <t>https://www.youtube.com/watch?v=heoMyS_hjm8</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=316780.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=321789.html</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>["https://fr.web.img4.acsta.net/img/87/b1/87b13594d74d6a0fe5bc1b5ae98acc87.jpg", "https://fr.web.img5.acsta.net/img/9b/27/9b2717b9517a0b1e09092932b9931850.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/48/79/4879231bf7df434ccefa260bf84fb18e.jpg", "https://fr.web.img2.acsta.net/img/06/47/0647937046e9709ff0b5a12f5af66696.jpg", "https://fr.web.img3.acsta.net/img/65/07/6507a80e00b779bd573a117ffb50cb59.jpg", "https://fr.web.img5.acsta.net/img/6d/64/6d641e15f7e1462ca5892078bb90c316.jpg", "https://fr.web.img5.acsta.net/img/69/b5/69b5410351d939cf5c005d68177db47c.jpg", "https://fr.web.img6.acsta.net/img/59/c4/59c4faa4bcbdbf003d6d30ecf546b632.jpg", "https://fr.web.img2.acsta.net/img/3f/d9/3fd9448d45fd39f1e5528ce6fef5de9d.jpg", "https://fr.web.img6.acsta.net/img/3d/a8/3da8c497a50cc952bb2b6da89f2095bd.jpg", "https://fr.web.img6.acsta.net/img/a5/ec/a5ecb292afd35323c0ba493853527eb1.jpg", "https://fr.web.img6.acsta.net/img/80/32/803246533fc9555b203272de850bede6.jpg", "https://fr.web.img4.acsta.net/img/5d/66/5d664316ddf74a92e69ea1f8bfb8051e.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Le garçon qui faisait danser les  collines</t>
+          <t>Gourou</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Georgi M Unkovski</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+          <t>Yann Gozlan</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/img/34/e6/34e60dd260546e67f467877cfb5316fc.jpg</t>
+          <t>https://fr.web.img3.acsta.net/c_310_420/img/70/e9/70e9dfd918886ca3ea4e1088f06f659c.jpg</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Ahmet, 15 ans, grandit au milieu des montagnes de Macédoine, où il garde les moutons de son père tout en prenant soin de son petit frère. Mais lui, ce qui le fait rêver, c’est la musique. Entre les attentes de son entourage et ses envies d’ailleurs, Ahmet pourra-t-il un jour suivre son propre chemin ?</t>
+          <t>Matt est le coach en développement personnel le plus suivi de France. Dans une société en quête de sens où la réussite individuelle est devenue sacrée, il propose à ses adeptes une catharsis qui électrise les foules autant qu'elle inquiète les autorités. Sous le feu des critiques, Matt va s'engager dans une fuite en avant qui le mènera aux frontières de la folie et peut-être de la gloire...</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Drame, Comédie, Musical</t>
+          <t>Thriller, Drame</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>99</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Pierre Niney, Marion Barbeau, Anthony Bajon, Christophe Montenez, Jonathan Turnbull, Raphaëlle Simon, Tracy Gotoas, Holt McCallany</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fJPl2vIVyQo</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000016927.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=328179.html</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>["https://fr.web.img4.acsta.net/img/51/fb/51fb8e6064ca7936232006c5e38d7bf9.jpg", "https://fr.web.img3.acsta.net/img/e2/31/e231cd9f9478af56c6927dfe4ca2501b.jpg"]</t>
+          <t>["https://fr.web.img3.acsta.net/img/9f/1d/9f1dbd266488613c10a426a974261b8c.jpg", "https://fr.web.img4.acsta.net/img/17/c6/17c6e2af9d1f11967aaaa2f1306b540b.jpg", "https://fr.web.img6.acsta.net/img/9a/7a/9a7a22f18891b552a20f418c87e1e687.jpg", "https://fr.web.img4.acsta.net/img/8c/19/8c1949acd4d427f4b9d91909697caca2.jpg", "https://fr.web.img6.acsta.net/img/f1/57/f157ec82c7710e95087f7e892512471f.jpg", "https://fr.web.img2.acsta.net/img/3b/8c/3b8cc41306419098a3af1f0ac5e363f7.jpg", "https://fr.web.img4.acsta.net/img/cd/49/cd49a9acf07e9a8c2402d874604c8ff7.jpeg", "https://fr.web.img6.acsta.net/img/ac/6a/ac6a7407004bee6c41d905d61ec8a19c.jpg", "https://fr.web.img2.acsta.net/img/93/00/9300f8b3ff1dba6e2e53a0708e08ce5f.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Affection, affection</t>
+          <t>Les légendaires</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2264,187 +2311,195 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Alexia Walther, Maxime Matray</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>Guillaume Ivernel</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/img/b0/82/b082ee3cbe7d6278acd9e6ac39d9d86b.jpg</t>
+          <t>https://fr.web.img4.acsta.net/c_310_420/img/2f/d5/2fd599857351d16d6bfdc4f2fefeb6c3.jpg</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Sur la Côte d'Azur, une adolescente disparaît le jour de son anniversaire. Géraldine, employée municipale, s'improvise alors détective. Personne n'a rien vu mais tout le monde a son mot à dire et Géraldine aura du mal à ne pas se laisser submerger par les potins, les théories et les croyances de chacun. Et ce n'est pas le retour inopiné de sa mère qui va lui faciliter la tâche. Une petite ville, c'est bien connu, c'est plein de petits crimes...</t>
+          <t>Les Légendaires, intrépides aventuriers, étaient les plus grands héros de leur temps. Mais suite à une terrible malédiction, les voilà redevenus... des enfants de 10 ans ! Danaël, Jadina, Gryf, Shimy et Razzia vont unir leurs pouvoirs pour vaincre le sorcier Darkhell et libérer leur planète de l’enfance éternelle…</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Comédie dramatique</t>
+          <t>Animation, Aventure, Fantastique</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>92</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Belgium, France</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Agathe Bonitzer, Nathalie Richard, Christophe Paou, Marc Susini, Clémentine Kaul-Surdez</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
+          <t>Roman Doduik, Esthèle Dumand, Elise Tilloloy, Thomas Sagols, Antoine Schoumsky, Damien Witecka, Arthur Raynal, Lila Lacombe</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>2025-08-13</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr"/>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pV1SWn1Ywh8</t>
+        </is>
+      </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000027142.html</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr"/>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=281028.html</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img4.acsta.net/img/10/ff/10fffdefacafe24db47b052863ddda62.jpg", "https://fr.web.img2.acsta.net/img/6f/07/6f0749c6a78b06af7232687f6896c672.jpg", "https://fr.web.img3.acsta.net/img/fe/59/fe59795cff026603ec6509286e65cae2.jpg", "https://fr.web.img6.acsta.net/img/f0/16/f016b8c3dc3203dc1f6b36353293eee8.jpg", "https://fr.web.img5.acsta.net/img/63/32/63320b85a89d275f1a5d0d9c780b500f.jpg", "https://fr.web.img5.acsta.net/img/1a/99/1a997d97ddaa1d8dab61bdccc071b3c5.jpg", "https://fr.web.img5.acsta.net/img/98/fa/98faf076534288ceb543108e73e3207d.jpg", "https://fr.web.img3.acsta.net/img/95/d0/95d0df4ac2e7cb287b1d136b1889e820.jpg", "https://fr.web.img6.acsta.net/img/83/8b/838bbdf0b368f01174af41af63eaffe4.jpg", "https://fr.web.img5.acsta.net/img/09/62/0962ef494b4d4977bafb691688c32bae.jpg", "https://fr.web.img2.acsta.net/img/ce/35/ce351996d5af1ff6e50d2998a7c7bd5d.jpg", "https://fr.web.img6.acsta.net/img/ed/7f/ed7ff9fd0290f42f9a31398fd5ab6aa7.jpg", "https://fr.web.img6.acsta.net/img/83/4a/834ac89d75abf72496de462950e27138.jpg", "https://fr.web.img5.acsta.net/img/3b/03/3b03d942d59f7242d36becaf8ef6eccf.jpg"]</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Un jour avec mon père</t>
+          <t>Soulèvements</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>VO</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Akinola Davies</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>Thomas Lacoste</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Documentaire</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/3a/17/3a17a236cc7eb6ab8b568027211f5224.jpg</t>
+          <t>https://fr.web.img4.acsta.net/c_310_420/img/c3/7a/c37aa39be9f24b3762c95b0d28a7f074.jpg</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Un jour avec mon père est un récit semi-autobiographique se déroulant sur une seule journée dans la mégalopole nigériane, Lagos, pendant la crise électorale de 1993. Un père tente de guider ses deux jeunes fils à travers l'immense ville alors que des troubles politiques menacent.</t>
+          <t>Un portrait choral à 16 voix, 16 trajectoires singulières, réflexif et intime d’un mouvement de résistance intergénérationnel porté par une jeunesse qui vit et qui lutte contre l’accaparement des terres et de l’eau, les ravages industriels, la montée des totalitarismes et fait face à la répression politique. Une plongée au cœur des Soulèvements de la Terre révélant la composition inédite des forces multiples déployées un peu partout dans le pays qui expérimentent d’autres modes de vie, tissent de nouveaux liens avec le vivant, bouleversant ainsi les découpages établis du politique et du sensible en nous ouvrant au champ de tous les possibles.</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Drame</t>
+          <t>Documentaire</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>93</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr"/>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
       <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>Avant-Première en Compétition, Festival de Cannes 2025: Caméra d'Or - Mention spéciale</t>
-        </is>
-      </c>
+      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr"/>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CC5sKvkiEVw</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000019740.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000027296.html</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>["https://fr.web.img2.acsta.net/img/9d/c8/9dc8a396dd653369fa38f649ce901b6c.jpg", "https://fr.web.img4.acsta.net/img/fc/c2/fcc2c65af7e14662b883a61b7ee9c6a4.jpg", "https://fr.web.img6.acsta.net/img/4c/13/4c136a85f4474c6e13b28af2437902c7.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/1b/9b/1b9b3ff33962144829022b709cd9ee29.jpg", "https://fr.web.img3.acsta.net/img/a8/d6/a8d605a0b6bf958ef499b1fe347caa9e.jpg", "https://fr.web.img6.acsta.net/img/b3/85/b385a9bc79a9b50b2e37726afabba547.jpg", "https://fr.web.img3.acsta.net/img/18/e8/18e87a4c19b442a9a594de55b3e42e6f.jpg", "https://fr.web.img4.acsta.net/img/9e/85/9e857d294d3501d642fbfebde5623275.jpg", "https://fr.web.img6.acsta.net/img/50/b1/50b18c73c1ab806956884548189929fa.jpg", "https://fr.web.img4.acsta.net/img/01/0b/010b514e411d69aac38a26e35f13befb.jpg", "https://fr.web.img2.acsta.net/img/5e/e0/5ee0a38037f945a584330baf7736faf4.jpg", "https://fr.web.img4.acsta.net/img/5e/92/5e924deac43ee2c8f58dc9042e799dc8.jpg", "https://fr.web.img6.acsta.net/img/d3/af/d3af16e8a3583e87ef91ddba434be514.jpg", "https://fr.web.img5.acsta.net/img/a3/22/a322fe516953faf65bbac4e0b40f7fae.jpg", "https://fr.web.img2.acsta.net/img/14/fe/14fe970670f30afc2c9aedb8c844f280.jpg", "https://fr.web.img6.acsta.net/img/83/25/8325aaf8312916c0f28c51308598b3b5.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>La maison des femmes</t>
+          <t>Les dimanches</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Melisa Godet</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Avant-Première</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+          <t>Alauda Ruíz de Azúa</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/c_310_420/img/d0/9f/d09ff1ec5ee43c6f7f17d6622d7422d0.jpg</t>
+          <t>https://fr.web.img2.acsta.net/c_310_420/img/18/71/18717c10a7a89df2cbf10f6584181ebd.jpg</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>À la Maison des femmes, entre soin, écoute et solidarité, une équipe se bat chaque jour pour accompagner les femmes victimes de violences dans leur reconstruction. Dans ce lieu unique, Diane, Manon, Inès, Awa et leurs collègues accueillent, soutiennent, redonnent confiance. Ensemble, avec leurs forces, leurs fragilités, leurs convictions et une énergie inépuisable.</t>
+          <t>Ainara, 17 ans, élève dans un lycée catholique, s'apprête à passer son bac et à choisir son futur parcours universitaire. A la surprise générale, cette brillante jeune fille annonce à sa famille qu'elle souhaite participer à une période d’intégration dans un couvent afin d'embrasser la vie de religieuse. La nouvelle prend tout le monde au dépourvu. Si le père semble se laisser convaincre par les aspirations de sa fille, pour Maite, la tante d’Ainara, cette vocation inattendue est la manifestation d'un mal plus profond …</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2454,55 +2509,55 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>118</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Spain, France</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Karin Viard, Lætitia Dosch, Oulaya Amamra, Eye Haïdara, Pierre Deladonchamps, Juliette Armanet, Laurent Stocker, Jean-Charles Clichet</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>Avant-Première</t>
-        </is>
-      </c>
+          <t>Blanca Soroa, Patricia López Arnaiz, Miguel Garcés, Juan Minujín, Mabel Rivera, Nagore Aranburu, Lier Alava, Noe Chiroque</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=yAwvKg9T47Q</t>
+          <t>https://www.youtube.com/watch?v=JTU224MnTUM</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000012019.html</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr"/>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000020167.html</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/3b/cb/3bcb5b416b32e7af3938ca6da2354161.jpg", "https://fr.web.img2.acsta.net/img/4a/2c/4a2ca4fa5c7c57f798c8a62840690b53.JPG", "https://fr.web.img5.acsta.net/img/37/e3/37e39954c8a41f30f2a7a4f57f208b7e.jpg", "https://fr.web.img6.acsta.net/img/a1/e2/a1e2fafa239c82277c9666a70113eabc.jpg", "https://fr.web.img5.acsta.net/img/7d/f3/7df35d0115cf51288fa6076afe776c8f.jpg"]</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Piro Piro</t>
+          <t>Les toutes petites créatures 2</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2513,126 +2568,98 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sung-ah Min</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>SCOL</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Ec Labastide Clermont</t>
-        </is>
-      </c>
+          <t>Lucy Izzard</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Tarif Unique 3 €</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>https://fr.web.img5.acsta.net/c_310_420/pictures/22/11/25/14/56/2428297.jpg</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Un ensemble de 6 films d’animation poétiques et sensibles où le talent de 2 de jeunes réalisatrices sud coréennes, Baek Miyoung et Min Sung-Ah, dévoile des univers aux couleurs pastel et chaleureuses. Des petits oiseaux tissent le lien entre ces films, dans lesquels on partage des instants de tendresse et d’humour. Programme :Koong ! Flap Flap :Quand un crocodile endormi rencontre un petit oiseau.A bird who loves a flower :L’histoire d’un oiseau qui aimait les fleurs.Ba-Lam :Le parcours initiatique d’un papillon bleu dont l’instinct lui dicte de suivre des fleurs en se laissant porter au gré du vent.Piro Piro :Piro Piro et Dalle sont 2 oiseaux. Le premier vient de la forêt, le second de la ville. Lorsqu’ils se rencontrent devant un magasin de fleurs, Piro Piro voudrait qu’ils s’envolent ensemble vers la forêt mais Dalle ne semble pas en état de voler...Dancing in the rain :Deux lapins dansent sous la pluie.The Newly Coming Seasons :La zone démilitarisée de Corée, créée suite à l’armistice du 27 Juillet 1953, est connue pour être un écosystème intact, loin de toute présence humaine. Mais coups de feux, incendies volontaires et intrusion de plantes étrangères font que de nombreux problèmes persistent entre le Nord et le Sud.</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Animation, Famille</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/70/e4/70e4bca25a2fa64e3574bcb887805ffe.jpg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>SCOL</t>
-        </is>
-      </c>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>2023-02-01</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=lwkHjaBZSHo</t>
-        </is>
-      </c>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=307792.html</t>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000037794.html</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>["https://fr.web.img6.acsta.net/pictures/22/09/09/13/04/3096825.jpg", "https://fr.web.img6.acsta.net/pictures/22/09/09/13/04/3081225.jpg", "https://fr.web.img6.acsta.net/pictures/22/09/09/13/03/3533794.jpg", "https://fr.web.img6.acsta.net/pictures/22/09/09/13/03/3519754.jpg", "https://fr.web.img4.acsta.net/pictures/22/09/09/13/03/3505714.jpg", "https://fr.web.img6.acsta.net/pictures/22/09/09/13/03/3491673.jpg", "https://fr.web.img6.acsta.net/pictures/22/09/09/13/03/3477633.jpg", "https://fr.web.img6.acsta.net/pictures/22/09/09/13/03/3463593.jpg", "https://fr.web.img6.acsta.net/pictures/22/09/09/13/03/3449553.jpg", "https://fr.web.img3.acsta.net/pictures/22/09/09/13/03/3433953.jpg", "https://fr.web.img3.acsta.net/pictures/22/09/09/13/03/3419913.jpg", "https://fr.web.img2.acsta.net/pictures/22/09/09/13/03/3404312.jpg"]</t>
+          <t>["https://fr.web.img6.acsta.net/img/20/9f/209f6648709f5ac9ac1b24d0b7300e8b.jpg", "https://fr.web.img6.acsta.net/img/e9/8d/e98d3ea0f91318eae342f1679376a5f5.jpg", "https://fr.web.img4.acsta.net/img/25/42/2542406b179eaa94973416ee53983824.jpg", "https://fr.web.img2.acsta.net/img/b4/be/b4bee561b2baf9b5ce48442ab59426f0.jpg", "https://fr.web.img6.acsta.net/img/95/4f/954f8835a08c41b04a5c95b7651eb3ef.jpg", "https://fr.web.img4.acsta.net/img/51/08/5108a7f9bd7a372c10b97486344b08c4.jpg"]</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Le mécano de la générale</t>
+          <t>Nurenberg</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>VO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Clyde Bruckman, Buster Keaton</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>SCOL</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+          <t>James Vanderbilt</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Coll Mandela Noé</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/pictures/17/05/19/16/07/057072.jpg</t>
-        </is>
-      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Le cheminot Johnnie Gray partage sa vie entre sa fiancée Annabelle Lee et sa locomotive, la Générale. En pleine Guerre de Sécession, il souhaite s'engager dans l'armée sudiste, mais celle-ci estime qu'il se montrera plus utile en restant mécanicien. Pour prouver à Annabelle qu'il n'est pas lâche, il se lance seul à la poursuite d'espions nordistes qui se sont emparés d'elle et de sa locomotive...</t>
+          <t>En 1948, le juge Haywood est envoyé à Nuremberg pour présider le procès de quatre magistrats allemands accusés de trop de complaisance à l'égard du régime Nazi. L'un d'eux, Janning, se renferme dans un silence méprisant et, en écartant les témoignages et les films sur les camps de concentration, dit qu'il n'a fait qu'appliquer la loi en vigueur...</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Action, Comédie</t>
+          <t>Drame, Histoire</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>179</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2642,119 +2669,1496 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Buster Keaton, Marion Mack, Glen Cavender, Jim Farley, Frederick Vroom, Frank Barnes, Charles Henry Smith, Joe Keaton</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>SCOL</t>
-        </is>
-      </c>
+          <t>Spencer Tracy, Richard Widmark, Maximilian Schell, Burt Lancaster, Marlene Dietrich, Judy Garland, Montgomery Clift, William Shatner</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1927-02-24</t>
+          <t>1961-12-20</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ZROzVhuddiI</t>
-        </is>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=108016.html</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>["https://fr.web.img3.acsta.net/medias/nmedia/18/65/53/29/18868528.jpg", "https://fr.web.img3.acsta.net/medias/nmedia/18/65/53/29/18868522.jpg", "https://fr.web.img4.acsta.net/medias/nmedia/18/65/53/29/18868532.jpg", "https://fr.web.img6.acsta.net/medias/nmedia/18/65/53/29/18868526.jpg", "https://fr.web.img3.acsta.net/medias/nmedia/18/65/53/29/18868519.jpg", "https://fr.web.img2.acsta.net/medias/nmedia/18/65/53/29/18868527.jpg", "https://fr.web.img6.acsta.net/medias/nmedia/18/65/53/29/18868517.jpg", "https://fr.web.img5.acsta.net/medias/nmedia/18/65/53/29/18868539.jpg", "https://fr.web.img6.acsta.net/medias/nmedia/18/65/53/29/18868520.jpg", "https://fr.web.img5.acsta.net/medias/nmedia/18/65/53/29/18868308.jpg", "https://fr.web.img4.acsta.net/medias/nmedia/18/65/53/29/18868538.jpg", "https://fr.web.img2.acsta.net/medias/nmedia/18/65/53/29/18868536.jpg", "https://fr.web.img6.acsta.net/medias/nmedia/18/65/53/29/18868534.jpg", "https://fr.web.img4.acsta.net/medias/nmedia/18/65/53/29/18868541.jpg", "https://fr.web.img2.acsta.net/medias/nmedia/18/65/53/29/18868530.jpg", "https://fr.web.img6.acsta.net/pictures/14/04/16/10/34/296957.jpg", "https://fr.web.img4.acsta.net/pictures/14/04/16/10/33/190777.jpg", "https://fr.web.img6.acsta.net/pictures/14/08/08/10/59/411069.jpg", "https://fr.web.img5.acsta.net/pictures/14/04/16/10/35/428400.jpg", "https://fr.web.img2.acsta.net/pictures/14/04/16/10/35/161355.jpg", "https://fr.web.img6.acsta.net/pictures/14/04/16/10/33/563814.jpg", "https://fr.web.img2.acsta.net/pictures/14/04/16/10/32/177456.jpg", "https://fr.web.img5.acsta.net/pictures/210/085/21008581_20130527145850575.jpg", "https://fr.web.img6.acsta.net/pictures/210/085/21008580_20130527145850341.jpg", "https://fr.web.img2.acsta.net/pictures/210/085/21008579_20130527145850106.jpg", "https://fr.web.img3.acsta.net/pictures/210/085/21008578_20130527145849841.jpg", "https://fr.web.img3.acsta.net/medias/nmedia/18/35/20/55/18389120.jpg", "https://fr.web.img4.acsta.net/medias/nmedia/18/35/20/55/18389121.jpg", "https://fr.web.img5.acsta.net/medias/nmedia/18/35/20/55/18389122.jpg", "https://fr.web.img6.acsta.net/medias/nmedia/18/35/20/55/18389123.jpg"]</t>
-        </is>
-      </c>
+          <t>https://www.youtube.com/watch?v=T3taV43-lGc</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Marsupilami JP famille</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Philippe Lacheau</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Séance EPHAD HANDI - Famille</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Tarif Unique 5 €</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>L'affaire Bojarski</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Aucun autre choix</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Park Chan-Wook</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://fr.web.img4.acsta.net/c_310_420/img/a4/52/a4527664f53d4cdc51dbaf628184aff1.jpg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Cadre dans une usine de papier You Man-su est un homme heureux, il aime sa femme, ses enfants, ses chiens, sa maison. Lorsqu’il est licencié, sa vie bascule, il ne supporte pas l’idée de perdre son statut social et la vie qui va avec. Pour retrouver son bonheur perdu, il n’a aucun autre choix que d’éliminer tous ses concurrents…</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Comédie, Thriller, Drame</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>139</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>South Korea, France</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Lee Byung-hun, Son Ye-jin, Park Hee-soon, Lee Sung-min, 염혜란, Seung-Won Cha, 김우승, 최소율</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HmIjLVScTCg</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000001960.html</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img4.acsta.net/img/f3/d4/f3d468179b397ececd43f1711bbc1a76.jpg", "https://fr.web.img6.acsta.net/img/60/57/605725c49daa9020d47c4ce10f25758a.jpg", "https://fr.web.img5.acsta.net/img/11/76/1176ff6544e51bdc85b65a25ae9f4bee.jpg", "https://fr.web.img5.acsta.net/img/34/9d/349dcb149bbeb77fab3cbdf72112b5cf.jpg", "https://fr.web.img3.acsta.net/img/1f/3a/1f3a26c88428a73486318b40a627d770.jpg", "https://fr.web.img6.acsta.net/img/16/27/162791ba5975e5bd6aeae70c26a57888.jpg", "https://fr.web.img4.acsta.net/img/36/e6/36e6055fcf5065eb0e303d5e1fb79f16.jpg", "https://fr.web.img6.acsta.net/img/20/43/2043b580d48745f6c512da8f8826b3bd.jpg", "https://fr.web.img5.acsta.net/img/98/62/986235bea13d02d81b9c69dce82abe97.jpg", "https://fr.web.img2.acsta.net/img/98/9d/989d2ca66bd7c50ea92e0687f7108618.jpg", "https://fr.web.img6.acsta.net/img/de/9f/de9f0f312b1363464f0179f405c388bb.jpg", "https://fr.web.img4.acsta.net/img/4e/ec/4eecf5368ac8628bc6f99a0c0831488b.jpg", "https://fr.web.img3.acsta.net/img/00/d8/00d81ae0aec94b670bce45db163e32af.jpg", "https://fr.web.img4.acsta.net/img/b6/22/b622dcefa6e2bc72b5d4ebb710477c8b.jpg", "https://fr.web.img5.acsta.net/img/21/ca/21cafa7467d6acbeea12fa5d317af65b.jpg", "https://fr.web.img3.acsta.net/img/0a/f6/0af620a91b2dd78a9ca9f56b066bf307.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Biscuit le chien fantastique</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>VF</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>CM2</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Jean-Paul Salomé</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>https://fr.web.img6.acsta.net/c_310_420/img/18/05/18059e8dd9bca2e516d41023cc08d9d1.jpg</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>Jan Bojarski, jeune ingénieur polonais, se réfugie en France pendant la guerre. Il y utilise ses dons pour fabriquer des faux papiers pendant l’occupation allemande. Après la guerre, son absence d’état civil l’empêche de déposer les brevets de ses nombreuses inventions et il est limité à des petits boulots mal rémunérés… jusqu’au jour où un gangster lui propose d’utiliser ses talents exceptionnels pour fabriquer des faux billets. Démarre alors pour lui une double vie à l’insu de sa famille. Très vite, il se retrouve dans le viseur de l’inspecteur Mattei, meilleur flic de France.</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Shea Wageman</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Ciné goûter, Jeune Public</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Tarif Unique 4,50 €</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/7b/09/7b095f309baf4441fc5966b2f217900e.jpg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Danny et son petit chien Biscuit sont les meilleurs amis du monde. Un jour, une magie mystérieuse donne à Biscuit des pouvoirs incroyables : il peut désormais parler et voler. Dès que quelqu’un a besoin de lui, il met son masque, enfile sa cape et s’élance dans le ciel pour aider : il est devenu un chien fantastique ! Biscuit a désormais deux passions : manger des tacos et sauver le monde. Mais Pudding, le chat du voisin, lui aussi doté de super-pouvoirs, rêve de faire régner les chats sur l’univers. Danny et Biscuit devront prouver qu’ensemble, rien ne peut les arrêter !</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Animation, Comédie, Famille</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Owen Wilson, Dawson Littman, Tabitha St. Germain, Sebastian Billingsley-Rodriguez, Rhona Rees, Anthony Bolognese, Caitlynne Medrek, Emily Delahunty</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VmxXMWGaDzQ</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000017117.html</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img3.acsta.net/img/cc/bb/ccbb0018fbe560c8535c07949d408025.jpg", "https://fr.web.img3.acsta.net/img/e7/ac/e7acc11655324629f86345607eafcf23.jpg", "https://fr.web.img2.acsta.net/img/f9/7b/f97bfe76e783f57e01a872b7c763cf47.jpg", "https://fr.web.img5.acsta.net/img/7f/c6/7fc688f605e3c9f8bb6fe9058bc80942.jpg", "https://fr.web.img5.acsta.net/img/67/0e/670e08bbd5558a2b53def24b58a59715.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Hamnet</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Chloé Zhao</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Ciné Jeunes du samedi 18h</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Adhérents 4 € - Autres 5 €</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://fr.web.img2.acsta.net/c_310_420/img/9a/f5/9af5f87b39938fec50f86c32c3d31b69.jpg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Angleterre, 1580. Un professeur de latin fauché, fait la connaissance d’Agnes, jeune femme à l’esprit libre. Fascinés l’un par l’autre, ils entament une liaison fougueuse avant de se marier et d’avoir trois enfants. Tandis que Will tente sa chance comme dramaturge à Londres, Agnes assume seule les tâches domestiques. Lorsqu’un drame se produit, le couple, autrefois profondément uni, vacille. Mais c’est de leur épreuve commune que naîtra l’inspiration d’un chef d’œuvre universel.</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
         <is>
           <t>Drame</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>United Kingdom, United States of America</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Jessie Buckley, Paul Mescal, Emily Watson, Joe Alwyn, Jacobi Jupe, Noah Jupe, Bodhi Rae Breathnach, Olivia Lynes</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Meilleure film dramatique et meilleure actrice Golden Globes 2026, Golden Globes 2026: Meilleur film dramatique, Meilleure actrice dans un drame</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xYcgQMxQwmk</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=315003.html</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/db/27/db27c1195bfb8835aef4671ac165e436.jpg", "https://fr.web.img3.acsta.net/img/ea/c4/eac4203c2df8347475f77ec8ce61d7ca.jpg", "https://fr.web.img6.acsta.net/img/7e/b8/7eb8bf6fa577347479dfd6347f103afb.jpg", "https://fr.web.img4.acsta.net/img/b0/3d/b03d7554c97c3f7ba8c880de57c35b31.jpg", "https://fr.web.img2.acsta.net/img/e0/f2/e0f2b4497faaf505ab30ecd733f2a531.jpg", "https://fr.web.img6.acsta.net/img/9a/fd/9afde980a6402b830c5007cc66e72aff.jpg", "https://fr.web.img5.acsta.net/img/ce/fe/cefe5da862eb8228d3bf79a068a9844a.jpg", "https://fr.web.img4.acsta.net/img/c0/41/c041a05c78908f57f777fb269f515979.jpg", "https://fr.web.img3.acsta.net/img/fd/f9/fdf917bfcee844d0fbd3ac41bba90997.jpg", "https://fr.web.img5.acsta.net/img/dc/88/dc886647f0301e242fd931547cd4d10e.jpg", "https://fr.web.img2.acsta.net/img/fc/d8/fcd8803be480fc3fd79f80b56597c9ba.jpg", "https://fr.web.img2.acsta.net/img/f1/de/f1deaf59daf5e4773c85bcf1702633d7.jpg", "https://fr.web.img2.acsta.net/img/5f/dc/5fdc64d7259e00568cfd5ab9344356b1.jpg", "https://fr.web.img3.acsta.net/img/19/5f/195f3ffc57720410317e2fb3d51ae61f.jpg", "https://fr.web.img2.acsta.net/img/b8/76/b876bf840dab929460f48ff0dac4d321.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>A pied d'œuvre</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Valérie Donzelli</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Achever un texte ne veut pas dire être publié, être publié ne veut pas dire être lu, être lu ne veut pas dire être aimé, être aimé ne veut pas dire avoir du succès, avoir du succès n'augure aucune fortune.
+ À Pied d’œuvre raconte l'histoire vraie d'un photographe à succès qui abandonne tout pour se consacrer à l'écriture, et découvre la pauvreté.</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Drame</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Bastien Bouillon, Marie Rivière, Virginie Ledoyen, André Marcon, Pauline Clément, Arthur Dupont, Émilie Caen, Quentin Dolmaire</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Gifr5NrMeBk</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Les légendaires</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Guillaume Ivernel</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://fr.web.img4.acsta.net/c_310_420/img/2f/d5/2fd599857351d16d6bfdc4f2fefeb6c3.jpg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Les Légendaires, intrépides aventuriers, étaient les plus grands héros de leur temps. Mais suite à une terrible malédiction, les voilà redevenus... des enfants de 10 ans ! Danaël, Jadina, Gryf, Shimy et Razzia vont unir leurs pouvoirs pour vaincre le sorcier Darkhell et libérer leur planète de l’enfance éternelle…</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Animation, Aventure, Fantastique</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Belgium, France</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Roman Doduik, Esthèle Dumand, Elise Tilloloy, Thomas Sagols, Antoine Schoumsky, Damien Witecka, Arthur Raynal, Lila Lacombe</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=pV1SWn1Ywh8</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=281028.html</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img4.acsta.net/img/10/ff/10fffdefacafe24db47b052863ddda62.jpg", "https://fr.web.img2.acsta.net/img/6f/07/6f0749c6a78b06af7232687f6896c672.jpg", "https://fr.web.img3.acsta.net/img/fe/59/fe59795cff026603ec6509286e65cae2.jpg", "https://fr.web.img6.acsta.net/img/f0/16/f016b8c3dc3203dc1f6b36353293eee8.jpg", "https://fr.web.img5.acsta.net/img/63/32/63320b85a89d275f1a5d0d9c780b500f.jpg", "https://fr.web.img5.acsta.net/img/1a/99/1a997d97ddaa1d8dab61bdccc071b3c5.jpg", "https://fr.web.img5.acsta.net/img/98/fa/98faf076534288ceb543108e73e3207d.jpg", "https://fr.web.img3.acsta.net/img/95/d0/95d0df4ac2e7cb287b1d136b1889e820.jpg", "https://fr.web.img6.acsta.net/img/83/8b/838bbdf0b368f01174af41af63eaffe4.jpg", "https://fr.web.img5.acsta.net/img/09/62/0962ef494b4d4977bafb691688c32bae.jpg", "https://fr.web.img2.acsta.net/img/ce/35/ce351996d5af1ff6e50d2998a7c7bd5d.jpg", "https://fr.web.img6.acsta.net/img/ed/7f/ed7ff9fd0290f42f9a31398fd5ab6aa7.jpg", "https://fr.web.img6.acsta.net/img/83/4a/834ac89d75abf72496de462950e27138.jpg", "https://fr.web.img5.acsta.net/img/3b/03/3b03d942d59f7242d36becaf8ef6eccf.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Promis le ciel</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Erige Sehiri</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/72/ba/72baef9032ae95ac8cf9be07f0cde8fe.jpg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Marie, pasteure ivoirienne et ancienne journaliste, vit à Tunis. Elle héberge Naney, une jeune mère en quête d'un avenir meilleur, et Jolie, une étudiante déterminée qui porte les espoirs de sa famille restée au pays. Quand les trois femmes recueillent Kenza, 4 ans, rescapée d'un naufrage, leur refuge se transforme en famille recomposée tendre mais intranquille dans un climat social de plus en plus préoccupant.</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Drame</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>France, Tunisia, Egypt</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Aïssa Maïga, Laëtitia Ky, Déborah Naney, Mohamed Grayaâ, Foued Zaazaa, Estelle Dogbo, Touré Blamassi, Sophie Tankou</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9F-U2tndiUo</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000006454.html</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/14/9f/149f6fcc8a302c7ea298d331efa5620d.jpg", "https://fr.web.img3.acsta.net/img/78/f1/78f16e1dbafb42446322d41ce4a2fca6.jpg", "https://fr.web.img2.acsta.net/img/29/eb/29eba2f15c17c7b55739027b37be608d.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Gourou</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Yann Gozlan</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://fr.web.img3.acsta.net/c_310_420/img/70/e9/70e9dfd918886ca3ea4e1088f06f659c.jpg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Matt est le coach en développement personnel le plus suivi de France. Dans une société en quête de sens où la réussite individuelle est devenue sacrée, il propose à ses adeptes une catharsis qui électrise les foules autant qu'elle inquiète les autorités. Sous le feu des critiques, Matt va s'engager dans une fuite en avant qui le mènera aux frontières de la folie et peut-être de la gloire...</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Thriller, Drame</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Pierre Niney, Marion Barbeau, Anthony Bajon, Christophe Montenez, Jonathan Turnbull, Raphaëlle Simon, Tracy Gotoas, Holt McCallany</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fJPl2vIVyQo</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=328179.html</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img3.acsta.net/img/9f/1d/9f1dbd266488613c10a426a974261b8c.jpg", "https://fr.web.img4.acsta.net/img/17/c6/17c6e2af9d1f11967aaaa2f1306b540b.jpg", "https://fr.web.img6.acsta.net/img/9a/7a/9a7a22f18891b552a20f418c87e1e687.jpg", "https://fr.web.img4.acsta.net/img/8c/19/8c1949acd4d427f4b9d91909697caca2.jpg", "https://fr.web.img6.acsta.net/img/f1/57/f157ec82c7710e95087f7e892512471f.jpg", "https://fr.web.img2.acsta.net/img/3b/8c/3b8cc41306419098a3af1f0ac5e363f7.jpg", "https://fr.web.img4.acsta.net/img/cd/49/cd49a9acf07e9a8c2402d874604c8ff7.jpeg", "https://fr.web.img6.acsta.net/img/ac/6a/ac6a7407004bee6c41d905d61ec8a19c.jpg", "https://fr.web.img2.acsta.net/img/93/00/9300f8b3ff1dba6e2e53a0708e08ce5f.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Les voyages de Tereza</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Gabriel Mascaro</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Cinélatino</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Cinélatino</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/a8/b9/a8b9fa641e4b57390f85e1efe2a0d0b0.jpg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Tereza a vécu toute sa vie dans une petite ville industrielle d’Amazonie. Le jour venu, elle reçoit l'ordre officiel du gouvernement de s’installer dans une colonie isolée pour personnes âgées, où elles sont amenées à « profiter » de leurs dernières années. Tereza refuse ce destin imposé et décide de partir seule à l'aventure, découvrir son pays et accomplir son rêve secret…</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Science Fiction, Drame</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Brazil, Mexico, Chile, Netherlands</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Denise Weinberg, Rodrigo Santoro, Miriam Socarrás, Adanilo, Rosa Malagueta, Clarissa Pinheiro, Dimas Mendonça, Daniel Ferrat</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Cinélatino, Berlinale 2025: Grand Prix du jury (Ours d'Argent)</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nFQEUuodCQ0</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000018687.html</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/07/04/070497f251d896cda1f60520a6d0fc54.jpg", "https://fr.web.img4.acsta.net/img/57/d3/57d3438239174ee61a0deb88160b00ea.jpg", "https://fr.web.img3.acsta.net/img/42/5d/425de28d088602fdd78202c4aab16839.jpg", "https://fr.web.img3.acsta.net/img/9d/ff/9dfffe21a51747bac25c9d1e50ee820a.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dreams</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Michel Franco</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Découverte</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>https://fr.web.img2.acsta.net/c_310_420/img/01/fe/01fe8bc3ac70f32388a4c0f2f812e251.jpg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Fernando, un jeune danseur de ballet originaire du Mexique, rêve de reconnaissance internationale et d’une vie meilleure aux États-Unis. Convaincu que sa maîtresse, Jennifer, une Américaine mondaine et philanthrope influente, l’aidera à réaliser ses ambitions, il quitte clandestinement son pays, échappant de justesse à la mort. Cependant, son arrivée vient bouleverser le monde soigneusement construit de Jennifer. Elle est prête à tout pour protéger leur avenir à tous deux, mais ne veut rien concéder de la vie qu'elle s'est construite.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Drame, Romance, Thriller</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Mexico, United States of America, United Kingdom</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Jessica Chastain, Isaac Hernández, Rupert Friend, Marshall Bell, Eligio Meléndez, Mercedes Hernández, Tatiana Ronderos, Bobby August Jr.</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=J6Al_zihrvw</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=320123.html</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img4.acsta.net/img/0d/1c/0d1cd828167f24891af42a411720a8be.jpg", "https://fr.web.img6.acsta.net/img/88/fd/88fd163059381b8cae2549df3e5e9e30.jpg", "https://fr.web.img6.acsta.net/img/01/ce/01ce1339cf23ecbf5bdea6194ed07fc9.jpg", "https://fr.web.img5.acsta.net/img/41/d2/41d2907555a93459497eb7b075f16b32.jpg", "https://fr.web.img2.acsta.net/img/a8/26/a826b9510da8463466852c141af624af.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Lol 2.0</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Lisa Azuelos</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://fr.web.img3.acsta.net/c_310_420/img/c4/54/c454690b912d2f827afd1c530d815186.jpg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Anne profite enfin de sa liberté après le départ de ses enfants. Mais tout bascule quand sa fille Louise, revient vivre chez elle après un échec professionnel et sentimental. Et comme une surprise n’arrive jamais seule, son fils Théo lui annonce qu’elle va devenir grand-mère ! Entre chocs générationnels, rêves en mutation et nouveaux élans amoureux… Anne comprend que la vie ne suit jamais tout à fait le plan prévu, et qu’à tout âge, on continue toujours d’apprendre à grandir.</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Comédie</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
         <is>
           <t>France, Belgium</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>Reda Kateb, Sara Giraudeau, Bastien Bouillon, Quentin Dolmaire, Pierre Lottin, Camille Japy, Lolita Chammah, Olivier Loustau</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Sophie Marceau, Thaïs Alessandrin, Françoise Fabian, Félix Moati, Alexandre Astier, Lou Lesage, Sandrine Bonnaire, Pierre Deladonchamps</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=2tyGg2W5NfE</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000024120.html</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/91/0c/910c9df46057596f7c75697ced84eefa.jpg", "https://fr.web.img3.acsta.net/img/b6/5a/b65abdfa3a24a32769eaa85105373ca4.jpg", "https://fr.web.img4.acsta.net/img/92/65/9265ce192a229f246430c135bae6be12.jpg", "https://fr.web.img4.acsta.net/img/cd/d5/cdd5ed3d51bafb6ec6b3ffafb4057b6d.jpg", "https://fr.web.img2.acsta.net/img/63/44/6344b9a3e80cf23b5b434333221468c6.jpg", "https://fr.web.img6.acsta.net/img/ab/b8/abb8eeba3fbcbe121af045fef1c39aca.jpg", "https://fr.web.img3.acsta.net/img/1d/48/1d48e8ac0dc355cf0a95757957ae76fb.jpg", "https://fr.web.img6.acsta.net/img/c7/34/c7342a1cffcbd824ea8b7db07a5c1ae2.jpg", "https://fr.web.img4.acsta.net/img/5e/c8/5ec8f9a5c2c2dda49e02c6190229cce6.jpg", "https://fr.web.img6.acsta.net/img/a1/31/a1314d5ea1ecefd608fcebf4bd68347f.jpg", "https://fr.web.img6.acsta.net/img/c0/c0/c0c07c78295184aecc47b9870b89627d.jpg", "https://fr.web.img4.acsta.net/img/49/be/49be1daf0d53e35466c50525a649edf9.jpg", "https://fr.web.img5.acsta.net/img/f3/8c/f38c33095b8afa91e7e63ff1b74b44a1.jpg", "https://fr.web.img4.acsta.net/img/cd/8d/cd8d6f6b9e616807904070250a3084fb.jpg", "https://fr.web.img2.acsta.net/img/0e/7c/0e7c4e425fc0b049d1ff4e68147fd6e8.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Super Charlie</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Jon Holmberg</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/f0/c9/f0c9c07f44b1e8dfd4f4793d81246491.jpg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Will âgé de 10 ans, a toujours rêvé de devenir un super-héros et de lutter contre le crime aux côtés de son père, policier. Mais, son rêve est brutalement remis en cause à la naissance de son petit frère Charlie. Non seulement ce nourrisson attire toute l’attention de la famille et au-delà, mais Will découvre que Charlie a des super-pouvoirs … Lorsqu’un super-vilain et un scientifique dérangé mettent en œuvre un plan diabolique, Charlie, coaché par son grand frère, va alors endosser le costume de super-héros pour sauver le monde !... Y parviendront-ils ?</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Animation, Famille, Aventure, Comédie, Fantastique</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Denmark, Sweden</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Orlando Wahlsteen, Silas Strand, Tuva Novotny, Sven Björklund, Joakim Jennefors, Ulla Skoog, Johan Rödin, Lily Wahlsteen</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zHJaTRoqmEA</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=326812.html</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img5.acsta.net/img/c0/66/c0664919c43cb4c8fe8a3b076a057927.jpg", "https://fr.web.img2.acsta.net/img/51/0b/510b034f5f6bd1da71aae528408e3401.jpg", "https://fr.web.img6.acsta.net/img/51/5d/515daf26bc81cbec87c4d058c0699bf1.jpg", "https://fr.web.img2.acsta.net/img/74/09/7409b263cc69e9c55718c4d29d38ff34.jpg", "https://fr.web.img6.acsta.net/img/85/2b/852ba5cdd9c51100baf3c3ba5f6c61a4.jpg", "https://fr.web.img6.acsta.net/img/45/1a/451a8e335d22a14dc3315a6e6671f199.jpg", "https://fr.web.img6.acsta.net/img/89/13/8913b1cf9700240e35f53ef740f096be.jpg", "https://fr.web.img3.acsta.net/img/7a/22/7a22cea3f50ab26aa3dc5739d1c18a8f.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Abel</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Elzat Eskendir</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Grand Prix et Prix de la critique Vesoul 2025</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Ciné discussion - Coup ce cœur</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Adhérents 4 € - Autres 5 €</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Grand Prix et Prix de la critique Vesoul 2025</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://fr.web.img2.acsta.net/c_310_420/img/a5/9d/a59db0f04640682ed57e6e0d153fe78e.jpg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Dans le tumulte post-soviétique du Kazakhstan en 1993, les fermes collectives sont démantelées et les propriétés sur le point d'être privatisées. Les dirigeants locaux ont depuis longtemps outrepassé leurs pouvoirs officiels, se partageant les ressources comme ils l’entendent. Abel, éleveur local, voudrait simplement sa part, mais la situation est plus complexe qu’il ne l’imaginait. Doit-il jouer le jeu de la corruption ou défendre ce qui lui paraît juste ?</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Famille, Drame</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Kazakhstan</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Yerlan Toleutay, Nurzhan Beksultanova, Alikhan Lepesbaev, Ulan Nusipali</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Grand Prix et Prix de la critique Vesoul 2025</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
         <is>
           <t>2026-01-14</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ArW4d3hKk60</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000014092.html</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>["https://fr.web.img4.acsta.net/img/15/d8/15d8fafca4998c253b2513d29f223350.jpg", "https://fr.web.img5.acsta.net/img/81/b3/81b30ddb0cecd137cedc5220f971c839.jpg", "https://fr.web.img6.acsta.net/img/b1/cf/b1cfe81aa1138030e212e9c701898bf6.jpg", "https://fr.web.img5.acsta.net/img/5a/cc/5acce5895b2080afc842c8d57340122c.jpg", "https://fr.web.img6.acsta.net/img/5d/1e/5d1e210d87c5045ba1d443e552d407f3.jpg", "https://fr.web.img6.acsta.net/img/b1/0f/b10f18819f1ccea971de115bc964d1d6.jpg"]</t>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000012048.html</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/0d/83/0d8360bdacfbb71b44bfdc8fb90ecf7f.jpg", "https://fr.web.img5.acsta.net/img/04/8e/048ebb38926740dfcfd073b3056a7b04.jpg", "https://fr.web.img4.acsta.net/img/8f/23/8f23909814dc0a2a580d89a815744c1c.jpg", "https://fr.web.img6.acsta.net/img/77/19/7719a44198a0cc7f2a1a2ed1d1e49913.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Maigret et le mort amoureux</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Pascal Bonitzer</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://fr.web.img4.acsta.net/c_310_420/img/59/d8/59d850a90c94bb8ebbbb22fbff9d4970.jpg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Le commissaire Maigret est appelé en urgence au Quai d’Orsay. Monsieur Berthier-Lagès, ancien ambassadeur renommé, a été assassiné. Maigret découvre qu’il entretenait depuis cinquante ans une correspondance amoureuse avec la princesse de Vuynes, dont le mari, étrange coïncidence, vient de décéder. En se confrontant aux membres des deux familles et au mutisme suspect de la domestique du diplomate, Maigret va aller de surprise en surprise...</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Policier</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>France, Belgium</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Denis Podalydès, Olivier Rabourdin, Micha Lescot, Laurent Poitrenaux, Irène Jacob, Manuel Guillot, Anne Alvaro, Julia Faure</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=G-_jyFNqjiY</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=325655.html</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img6.acsta.net/img/4c/4d/4c4dc3d77c2856f1326750e92055846b.jpg", "https://fr.web.img6.acsta.net/img/60/8a/608a37aacde1ea9c31e956ac83572fe0.jpg", "https://fr.web.img4.acsta.net/img/3e/0a/3e0aae1da4936eac025c4c097c0b2422.jpg", "https://fr.web.img6.acsta.net/img/e1/6e/e16e92bc9774d5ec304ae243afece809.jpg", "https://fr.web.img6.acsta.net/img/de/68/de688f3fa92fda9440f9423a8688cbe3.jpg", "https://fr.web.img2.acsta.net/img/33/5b/335b2eef6f1ae0101537081120fedf33.jpg", "https://fr.web.img2.acsta.net/img/68/56/6856f89d96ed0a1a1f56a8fc639032c1.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tafiti</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Nina Wels</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Jeune Public</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Tarif Unique 4,50 €</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://fr.web.img5.acsta.net/c_310_420/img/e7/ff/e7ffdee0f33865e434c017c192af11ac.jpg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Lorsque Tafiti, un jeune suricate, rencontre Mèchefol, un potamochère aussi sympathique qu’exubérant, il sait qu’ils ne pourront jamais devenir amis. En effet, la vie dans le désert est pleine de dangers et Tafiti a toujours respecté la règle essentielle de survie chez les suricates : il ne faut jamais se lier aux étrangers. Mais lorsque son grand-père est mordu par un serpent venimeux, Tafiti n’a pas le choix. Il doit partir à la recherche d’une fleur légendaire qui guérit de tous les maux, mais qui pousse au-delà des vastes étendues brûlantes du désert. Une quête périlleuse que Tafiti décide d’affronter seul. Mais c’est sans compter sur Mèchefol, bien décidé à accompagner son nouveau meilleur ami dans cette aventure, qu’il le veuille ou non…</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Animation, Famille, Aventure</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Cosima Henman, Steve Hudson, Bürger Lars Dietrich, Thomas Schmuckert, Dela Dabulamanzi, Simon Werner, Dustin Semmelrogge, Simone Cohn-Vossen</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=0AG59XQEhbA</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=327254.html</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img5.acsta.net/img/19/77/1977bdc7a0058cac90b8d00732caf0ca.jpg", "https://fr.web.img4.acsta.net/img/52/e6/52e62dd9215f23f1e25d326ba6b7a5fa.jpg", "https://fr.web.img2.acsta.net/img/e5/7e/e57edcf31ace74fb0a0f6f4de3be14cd.jpg", "https://fr.web.img6.acsta.net/img/aa/9f/aa9ff537ce0c29024615907c2622e4eb.jpg", "https://fr.web.img2.acsta.net/img/e5/8e/e58e207ab8bc2ac27ba7fec7da0c3696.jpg", "https://fr.web.img6.acsta.net/img/0a/ff/0aff7a5c96e70c97623d4098cfe9e51b.jpg", "https://fr.web.img4.acsta.net/img/83/73/837380da5f0906bbc4ddd94b380822c0.jpg", "https://fr.web.img3.acsta.net/img/65/3e/653e66af639a0e783b18aecde51ff7f3.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Les enfants de la Résistance</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Christophe Barratier</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Famille, Jeune Public</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/0f/58/0f58892693cc868f4c0caf21614954cf.jpg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Pendant l’occupation allemande durant la Seconde Guerre mondiale, François, Eusèbe et Lisa, trois enfants courageux, se lancent dans une aventure secrète : résister aux nazis en plein cœur de la France. Sabotages, messages cachés et évasions périlleuses, ils mènent des actions clandestines sous le nez de l’ennemi. L’audace et l’amitié sont leurs seules armes pour lutter contre l’injustice.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Drame, Historique, Aventure, Famille</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>France, Belgium</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Artus, Gérard Jugnot, Pierre Deladonchamps, Julien Arruti, Oscar Boissière, Leslie Medina, Julien Pestel, Vanessa Guide</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-2v2vWrUwcA</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000006174.html</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img2.acsta.net/img/8a/42/8a4292a470667f8315381e42f336d546.jpg", "https://fr.web.img2.acsta.net/img/cc/c7/ccc7fb7e24f2235353ddf413eb3b8734.jpg", "https://fr.web.img4.acsta.net/img/f4/15/f4153f99f16722bd823824a193194ef2.jpg", "https://fr.web.img5.acsta.net/img/f4/8f/f48f09cfc47da3cd5ac0478fc59f009c.jpg", "https://fr.web.img2.acsta.net/img/e2/f9/e2f9eb754cbec5fa08ec375ab52c1309.jpg", "https://fr.web.img5.acsta.net/img/a8/5f/a85f6763e4eb13807ebf8c3a67dd508e.jpg", "https://fr.web.img4.acsta.net/img/31/ca/31cab79941ff24e2744c2e49315c7573.jpg", "https://fr.web.img5.acsta.net/img/1a/c1/1ac144fe2f6c4df6d2656c9998eab111.jpg"]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Le mystérieux regard du flamant rose</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>VO</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Diego Cespedes</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Cinélatino</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Coup de cœur</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Cinélatino</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/a8/e5/a8e526e77f84a98e7a6d5dac7ba8e7f6.jpg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Début des années 1980, dans le désert chilien. Lidia, 11 ans, grandit au sein d’une famille flamboyante qui a trouvé refuge dans un cabaret, aux abords d’une ville minière. Quand une mystérieuse maladie mortelle commence à se propager, une rumeur affirme qu’elle se transmettrait par un simple regard. La communauté devient rapidement la cible des peurs et fantasmes collectifs. Dans ce western moderne, Lidia défend les siens.</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Drame</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Chile, France, Spain, Belgium, Germany</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Tamara Cortés, Matías Catalán, Paula Dinamarca, Claudia Cabezas, Luis Dubó, Andrés Almeida, Felipe Ríos, Vicente Caballero</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Cinélatino, Festival de Cannes 2025: Prix Un Certain Regard</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=69S7bBUiBN8</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=298832.html</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img2.acsta.net/img/82/90/82907cef76c8a8ed8ab5d99aab91f455.jpg", "https://fr.web.img2.acsta.net/img/44/85/44856197be75652c1527a3fcfc6a3d8b.jpg", "https://fr.web.img4.acsta.net/img/51/ab/51abdf1a07284b46031cdcda424d365e.jpg", "https://fr.web.img3.acsta.net/img/d3/3f/d33f7ebf1c5fefeb979bbd0439b138d0.png"]</t>
         </is>
       </c>
     </row>

</xml_diff>